<commit_message>
Invoice Refresh: portal cases closed, blockers ticketed, learnings recorded
120 cases executed: 110 Passed, 6 Failed, 4 Blocked.
- C44951, C45175 Passed; C44952 Failed on clause 4 -> SV-9797 (spec correction)
- C44902 -> SV-9799, C44907 -> SV-9800, C44916 -> SV-9710 (commented)
- C44951/C44952/C45175 preconditions now carry the real portal route
- L29-L32 recorded; playbook gains the customer-portal section

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWbxRKg4riKCp3gpbbwYzA
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Execution-Results_2026-09-07.xlsx
+++ b/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Execution-Results_2026-09-07.xlsx
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -565,6 +565,288 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>C-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>TestRail link</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Case title</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>What was observed</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>What still needs doing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>C44917</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44917</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Order Reference Fields</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Work Order field hides when it equals the document number's trailing digits</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>VERDICT FLIPPED after Chris Ward's ruling on SV-9770 (7 September 2026, spec live page v57). S3-N1 has been rewritten and the trailing-digits comparison is retired: the Work Order field is now hidden in exactly two cases - the document has no work order behind it, or the work order number and the document number are character-for-character identical as whole strings - and shown in every other case. Re-checked live on the current build: work order 'S-32136', document 'INV-S2-32136'. The two strings are NOT identical, so under the rewritten rule the field must SHOW. The build still hides it - the order-reference row renders only 'Customer PO 9989', 'Authorizer Savannah Tran', 'Terms Net 7'.</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Nothing further - the rule now has a definite answer and the build does not meet it. ALREADY TRACKED - SV-9642, 'Work Order chip hidden when the WO number does not match the document number', Story Defect under SV-9142 (Story 3), status Code Review, raised by Mudassir. Chris linked it to SV-9770 and said whichever is picked up first should close both. NO new ticket raised. THE CASE ITSELF NOW NEEDS REWRITING: its title and all three clauses describe the retired trailing-digits rule. It should be re-authored against the new S3-N1 (two enumerated hide cases) and the new S3-R10 (the field shows the work order number exactly as it appears on the work order, no prefix added, no reformatting - 'S-32136' reads 'S-32136' on a document numbered 'INV-S2-32136'). That is authoring work, not this lane's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>C44926</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44926</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Asset Section</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Unit, Plate, Mileage and Eng Hrs each hide when empty</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Unit and Plate follow the rule; Mileage and Eng Hrs do not. Seeded an asset with none of the four set and rendered the Estimate for work order S2-32226, where the live record reads mileage=null and engine_hours=null. The document hides UNIT and PLATE correctly - no label, no empty value - but prints 'MILEAGE 0' and 'ENG HRS 0' for the two fields that have no value at all. S4-N1 requires all four to be hidden when empty. Reproduced on a second record, INV-S2-32225, and on the invoices for S2-32219 and S2-32220, all of which print 'ENG HRS 0' against a null reading. Clause 2 holds: fields that do have values still show (INV-S2-32136 prints MILEAGE 45 and ENG HRS 9,987).</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>ALREADY REPORTED - SV-9680, 'Asset band prints Mileage 0 and Eng Hrs 0 for an asset with no recorded values', status Code Review. No new ticket raised. The fix has not reached staging build v26.35.9-9812433.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>C44935</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44935</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Work Section</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Line footer shows Labor, Parts and Line total with the divider rule</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Clauses 1, 3 and 4 hold: every work line carries a footer, the Labor/Parts figures follow their summarize and price settings, and the vertical divider before 'Line total' behaves as specified. CLAUSE 2 FAILS. On work order S-32136 line 01 (labour 2 x $149.95 = $299.90) a line-level fee of $25.00 was added (scope labor_line). The document renders the adjustment row correctly under the line as '↳ ZZAUTOTEST Line Fee  $25.00', but the line footer still reads 'Labor $299.90' and 'Line total $299.90'. S5-R9 requires the Labor and Parts figures to be the line's own totals AFTER its line-level fees and discounts, with Line total their sum - so both should read $324.90. The Design Document computes it that way in its own script: setTxt('j2-labor', money(599.80 + L + F)) and setTxt('j2-line', money(1004.88 + net)), with the comment that only the SUMMARY rows stay gross. The summary does add the fee once, under Adjustments &gt; Labor, so the customer is charged $324.90 for a line the document totals at $299.90.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Re-verdicted. The earlier Passed was reached on a work order that carried no adjustments, so clause 2 was never exercised. Defect candidate raised to the QA lead; nothing filed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>C44952</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44952</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Paid Banner, Payments and Balance</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Each banner payment shows its labeled fields and conditional fees/marker</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Clauses 1, 2, 3, 5 and 6 all PASS, observed live in the customer portal on staging. (1) Labels read exactly 'Date / Time', 'Paid By', 'Method', 'Invoice Amount', 'Total Charged'. (2) On the batch payments (S-32264 and S-12725) the label reads exactly 'Total Charged (Batch)' and carries the whole batch - S-32264 shows Invoice Amount CA$406.09 against Total Charged (Batch) CA$14,230.01. (3) 'Convenience Fee' shows on every payment that carried one; 'Late Fee' shows only on S-12725, whose payment carried a CA$4.73 late fee, and is absent everywhere the late fee was zero. (5) On S-32220, which has one single payment then one batch payment, the markers read 'Payment 1 of 2' and 'Payment 2 of 2 - Batch' with a middle dot, exactly as spec v57 S8-R9 writes it. (6) 'Date / Time' read 'Sep 7, 2026 - 10:23 AM MDT' - date, then 12-hour time with the shop timezone abbreviation.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>FAILS clause 4. 'Remaining Balance' never appears. Tested on four invoices where the balance immediately after a listed payment was greater than $0.00: S-32263 ($306.09 after payment 1 of 2), S-32220 ($150.23 after payment 1 of 2), S-32052 ($7.45 after the portal payment, still PARTIALLY PAID) and the partially paid state of S-32263. The string 'Remaining Balance' does not exist anywhere in the portal front end: all 133 JS assets in the portal build manifest were downloaded and searched, zero occurrences. The banner is rendered entirely client-side by PreviewInvoice-DQmgXtBb.js - the server's own invoice HTML carries none of the banner strings. PRODUCTION carries the same code: portal.shopview.com serves PreviewInvoice-DQmgXtBb.js byte-identical to staging (sha256 626a1d5723ef32a340fc78161caad3a6b4153313dd7f0e97e49babac1d4c1c77). Because S8-R8 states the banner is 'Behavior already in production, restated unchanged' and S8-R9 is not marked net-new, the spec's own precedence rule applies: a non-net-new rule that disagrees with production is amended to describe production. The finding is therefore raised as a SPEC CORRECTION, not as a build defect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>C44970</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44970</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Credit Invoice</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Credit Invoice shows the disclaimer and standard signature area</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Confirmed as a real defect and filed as SV-9790. Re-verified on two credits created minutes apart on the same account, same shop, same day. CM-4357 (raised with no originating invoice): NO disclaimer at all - the column beside the totals, where it belongs, is blank, and the document runs from the credit line straight to the signature lines. CM-4358 (raised from invoice INV-S-32262): the SAME shop disclaimer prints in full in that same column. The only structural difference between the two documents is the INVOICE NUMBER column. Clause 2 passes on both: all three signature lines print. Ruled out per the toggle discipline: the disclaimer IS configured (1,036 characters at Administration &gt; Settings &gt; Invoice, and CM-4358 proves it renders), and there is no per-document switch for it - the gear-icon toggles cover only labor/part display and the two summarize options. Reproduced on eight further no-invoice credits earlier the same day.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>FILED AS SV-9790 (Story Defect, Medium, parent SV-9150) on the QA lead's instruction. Duplicate search run first over 'disclaimer', 'credit memo' and 'Credit Invoice' - nothing covers it; SV-8115 is a Done layout issue from an earlier build. The case's own text predicts this as outcome (2), which is why it was not filed on the first pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>C44974</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44974</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Document Visual Standard</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Typography uses Inter with the specified weights</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>The typeface in the generated PDF is NOT Inter. Every embedded font on every document type is DejaVu Sans: subsets 'XKQQSR+DejaVu-Sans' and 'UWGIWA+DejaVu-Sans-Bold', and nothing else - confirmed on the Invoice (INV-S2-32136), the Estimate (EST-S2-32136), the deposit-paid Invoice (INV-S2-32217) and the Credit document (CM-4347). The template's own CSS asks for Inter ('Inter', -apple-system, 'Segoe UI', Roboto, sans-serif) and its comment asserts 'Inter ships in the WeasyPrint image (Phase 3)', so the PDF pipeline is falling back to WeasyPrint's default face. Consequence for clause 2: only two faces are embedded, regular and bold, so the 400/600/700/800 ladder the spec and the Design Document require collapses to regular-or-bold - 600, 700 and 800 are indistinguishable on paper.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Clause 1's screen half (whether the in-app preview renders Inter) was not measured; the failure is proven for PDF output, which is enough to fail the case since the rule requires the two to match line for line. Defect candidate raised to the QA lead with the design and spec references; nothing filed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -622,148 +904,148 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>C44926</t>
+          <t>C44902</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44926</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44902</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Asset Section</t>
+          <t>Masthead and Letterhead</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Unit, Plate, Mileage and Eng Hrs each hide when empty</t>
+          <t>Shop logo shows when set; nothing (no placeholder) shows when unset</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Unit and Plate follow the rule; Mileage and Eng Hrs do not. Seeded an asset with none of the four set and rendered the Estimate for work order S2-32226, where the live record reads mileage=null and engine_hours=null. The document hides UNIT and PLATE correctly - no label, no empty value - but prints 'MILEAGE 0' and 'ENG HRS 0' for the two fields that have no value at all. S4-N1 requires all four to be hidden when empty. Reproduced on a second record, INV-S2-32225, and on the invoices for S2-32219 and S2-32220, all of which print 'ENG HRS 0' against a null reading. Clause 2 holds: fields that do have values still show (INV-S2-32136 prints MILEAGE 45 and ENG HRS 9,987).</t>
+          <t>Clause 1 verified: when a logo is set the masthead shows it - a 2208x480 JPEG, 408,254 bytes, placed centrally in the masthead at x=228.8-342.8 on every document rendered this pass.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>ALREADY REPORTED - SV-9680, 'Asset band prints Mileage 0 and Eng Hrs 0 for an asset with no recorded values', status Code Review. No new ticket raised. The fix has not reached staging build v26.35.9-9812433.</t>
+          <t>Clause 2 - that nothing shows when no logo is set. The search is now exhaustive and the state cannot be produced. (1) The logo is ORGANISATION-level, not per-location: no logo field exists on any location record, so the case's precondition of one shop with a logo and one without cannot exist. (2) The UI offers no removal: the only control is a pencil overlay on the image at Administration &gt; Settings &gt; Organization, and it opens a file picker (accept '.jpg, image/*') - replace only. (3) The API has no removal either. The read route GET /api/organization/organization-details/logo answers 405 'Allow: GET' to DELETE. The write route was found by driving the picker with a request listener - POST /api/organization/organization-details/upload-logo - and it answers 405 to DELETE. Guessed removal routes remove-logo and delete-logo are both 404 on POST and DELETE. Raised as SV-9799 (QA blocker — a shop logo can be added or replaced but never removed). Re-proved today from a fourth direction: `organization/organization-details/change`, the only organisation-update endpoint the app has, does not carry a logo field at all (its contract is company name, state/province, city, address 1, postal code, telephone, email, tax code, country code), so there is no remove path even at the API. Organisations created fresh DO start with no logo — the staging estate has ~100 E2E-Bootstrap organisations whose logo is null — but ShopView exposes no way to switch into another organisation, and the Team Tools admin (staging.teamtools.portal.shopview.com) needs its own login. Clause 1 (a logo, when set, shows) stays verified.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>C44935</t>
+          <t>C44907</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44935</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44907</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Work Section</t>
+          <t>Masthead and Letterhead</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Line footer shows Labor, Parts and Line total with the divider rule</t>
+          <t>Masthead identity fields each hide when empty</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Clauses 1, 3 and 4 hold: every work line carries a footer, the Labor/Parts figures follow their summarize and price settings, and the vertical divider before 'Line total' behaves as specified. CLAUSE 2 FAILS. On work order S-32136 line 01 (labour 2 x $149.95 = $299.90) a line-level fee of $25.00 was added (scope labor_line). The document renders the adjustment row correctly under the line as '↳ ZZAUTOTEST Line Fee  $25.00', but the line footer still reads 'Labor $299.90' and 'Line total $299.90'. S5-R9 requires the Labor and Parts figures to be the line's own totals AFTER its line-level fees and discounts, with Line total their sum - so both should read $324.90. The Design Document computes it that way in its own script: setTxt('j2-labor', money(599.80 + L + F)) and setTxt('j2-line', money(1004.88 + net)), with the comment that only the SUMMARY rows stay gross. The summary does add the fee once, under Adjustments &gt; Labor, so the customer is charged $324.90 for a line the document totals at $299.90.</t>
+          <t>Clause 2 holds: fields that have values do show, on every document produced this pass. Clause 1's state cannot exist in the product, now proven from two directions. (a) AT CREATION: Administration &gt; Locations &gt; New Location refuses to save without them - attempting a location with only a name and shop id returns 'Address is a required field' and 'City is a required field', and supplying those two then returns 'State/Province is a required field', 'ZIP/Postal code is a required field' and 'Telephone is a required field' (plus Country and Timezone). Every one of the five masthead identity fields is mandatory. (b) AT EDIT: clearing all four editable ones on an existing location and saving reports no error but does not persist - the record reads back unchanged, verified by clearing, saving, re-reading, then restoring and re-reading again.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Re-verdicted. The earlier Passed was reached on a work order that carried no adjustments, so clause 2 was never exercised. Defect candidate raised to the QA lead; nothing filed.</t>
+          <t>Clause 1 - each missing masthead field being hidden with no blank line left. Raised as SV-9800 (QA blocker — all five masthead identity fields are mandatory). Re-proved through the UI today: Administration &gt; Locations &gt; New location, name only, Save &amp; Close, marks Address 1, City, State/Province, Country, ZIP/Postal Code, Timezone and Telephone red as required even though only Name carries the asterisk. Clause 2 (fields with values show normally) stays verified on every document produced this pass.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>C44970</t>
+          <t>C44916</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44970</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44916</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice</t>
+          <t>Order Reference Fields</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice shows the disclaimer and standard signature area</t>
+          <t>Approval Code field shows the integrated-billing approval code</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Outcome (2) in the case reproduces exactly. On the credit raised from an invoice (CM-4355, status table carrying 'INVOICE NUMBER  INV-S-32220') the full disclaimer prints just above the three signature lines - that half passes. On every credit with no invoice number (CM-4348, CM-4350, CM-4351, CM-4352, CM-4353, CM-4354, CM-4324, CM-4347 - eight documents) NO disclaimer prints at all, only 'CUSTOMER SIGNATURE / PRINTED NAME / DATE'. The shop does have one configured, which CM-4355 proves. Clause 2 passes on all nine documents.</t>
+          <t>Integrated billing IS configured on this organisation - Administration &gt; IBS carries a remit-to payee (Punta Gorda Truck Service &amp; Repair) and customers carry IBS account numbers, for example East Moline Diesel Repair with company_ibs 875790. But no work order has ever been issued an approval code: ibs_approval_code is null on all 100 work orders read live at Staging Heavy Duty - 9919, and null on S-17466 too, which belongs to an IBS customer. There is also no way to seed one - the app exposes no route that sets an approval code (the only 'approval' routes are createApprovalRequest and checkApprovalRequestExists, which are the customer work-approval feature, and every IBS route is about batches and payments: create-batch, list-batches, batch-export, list-payments, list-transactions, payment, reverse-payment).</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Marked Failed per the case's own instruction; it fails in exactly the way described, so nothing new is raised. No Jira ticket exists for it - it is reported here with its C-id per the standing rule that a pass ends in a runnable test, not a defect.</t>
+          <t>Both clauses - the Approval Code showing in its own field labeled exactly 'Approval Code', and it no longer appearing under the 'Authorizer' label. Maps to the EXISTING ticket SV-9710 (IBS approval cannot be requested on QA — Approval Code chip (S3-R4) unverifiable), which was Open before this pass; a comment was added recording that it reproduces on staging. Staging is one level worse than QA: the IBS integration is not connected at all on this organisation (Administration &gt; IBS: isConfigured false, isActive false, baseUrl null) and all three shop locations have an empty IBS Location ID. No new ticket was raised because SV-9710 already carries this.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>C44974</t>
+          <t>C45275</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44974</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45275</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Document Visual Standard</t>
+          <t>Authorizer Entry (Work Order)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Typography uses Inter with the specified weights</t>
+          <t>Changing the customer clears the Authorizer; changing only the contact does not</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>The typeface in the generated PDF is NOT Inter. Every embedded font on every document type is DejaVu Sans: subsets 'XKQQSR+DejaVu-Sans' and 'UWGIWA+DejaVu-Sans-Bold', and nothing else - confirmed on the Invoice (INV-S2-32136), the Estimate (EST-S2-32136), the deposit-paid Invoice (INV-S2-32217) and the Credit document (CM-4347). The template's own CSS asks for Inter ('Inter', -apple-system, 'Segoe UI', Roboto, sans-serif) and its comment asserts 'Inter ships in the WeasyPrint image (Phase 3)', so the PDF pipeline is falling back to WeasyPrint's default face. Consequence for clause 2: only two faces are embedded, regular and bold, so the 400/600/700/800 ladder the spec and the Design Document require collapses to regular-or-bold - 600, 700 and 800 are indistinguishable on paper.</t>
+          <t>Nothing to verify against. The case has a precondition but its Steps and its Expected Results are both EMPTY - read raw from TestRail, custom_steps is null and custom_expected is null. There is no stated behaviour to test.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Clause 1's screen half (whether the in-app preview renders Inter) was not measured; the failure is proven for PDF output, which is enough to fail the case since the rule requires the two to match line for line. Defect candidate raised to the QA lead with the design and spec references; nothing filed.</t>
+          <t>Unchanged and unchangeable by us: created_by = 1 (Vladimir Tomovic), and its Steps and Expected Results are both empty in TestRail. Standing rule 38 keeps his cases hands-off, so this is reported and left exactly as it is. Its author needs to supply steps and expected results before it can be run.</t>
         </is>
       </c>
     </row>
@@ -772,13 +1054,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -830,12 +1112,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>C44902</t>
+          <t>C44901</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44902</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44901</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -845,34 +1127,30 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Shop logo shows when set; nothing (no placeholder) shows when unset</t>
+          <t>Masthead shows the shop location's full identity details</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 IS verified: when the shop has a logo set, the masthead shows it. The logo is an embedded 2208x480 image placed centrally in the masthead at x=228.8-342.8, y=70.4-95.2, present on every document rendered this pass.</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Clause 2 - that nothing at all shows when no logo is set. No logo control could be found anywhere in the product: it is not on Administration &gt; Locations (the Edit Location dialog has no logo field and no file input), not on the New Location dialog, and not on Administration &gt; Settings, whose Organization tab holds only company name, address, telephone, email and Tax ID and whose Invoice tab holds only the nine display toggles and the disclaimer. To finish it: find where the shop logo is uploaded - it may be an organisation-level setting not exposed in this build's admin screens - remove it for a test location, and render a document to confirm the masthead shows no logo and no placeholder box, image or 'no logo' text in its place.</t>
-        </is>
-      </c>
+          <t>All five identity values match the shop record byte-for-byte: name 'Staging Heavy Duty - 9919', '9919 Shepard Road SE', 'Calgary, Alberta', 'T2C 4M5', '(403) 523 - 0488' (GET /api/workplaces).</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>C44907</t>
+          <t>C44903</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44907</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44903</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -882,689 +1160,263 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Masthead identity fields each hide when empty</t>
+          <t>Document label names the type before the number on each document</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>The state cannot be created in the product. On Administration &gt; Locations &gt; Staging Heavy Duty - 9919 the address, city, postal code and telephone fields clear in the form and 'Save' reports no error, but the record is unchanged afterwards: reading the location back gives '9919 Shepard Road SE / Calgary / Alberta / T2C 4M5 / (403) 523 - 0488' exactly as before. Verified by clearing all four, saving, and reading the live record - identical - then restoring and re-reading, also identical. The same silent no-op affects the organisation Tax ID (see C44958), so these identity fields appear to be treated as mandatory even though no validation message is shown. Clause 2 holds trivially: fields that have values do show, on every document produced this pass.</t>
+          <t>All three document labels now observed: 'Estimate: EST-S2-32136', 'Invoice: INV-S2-32136' and 'Credit: CM-4347'. In each the type word precedes the number and the number carries its type prefix (EST- / INV- / CM-).</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - each missing masthead field being hidden with no blank line left. The empty state could not be produced. To finish it: have a location saved with one or more of street address, city, state/province, postal code or telephone genuinely blank (a developer or a direct data change may be needed, since the Locations form will not persist an empty value), then render any document at that location and check no blank line or empty label is left. The environment was left exactly as found - the location record was re-read after restoring and matches the original in every field.</t>
+          <t>The Invoices LIST renders the credit as 'CM2-4347', but the DOCUMENT reads 'CM-4347' - the document is what this case asserts, and it is correct.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>C44916</t>
+          <t>C44904</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44916</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44904</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Order Reference Fields</t>
+          <t>Masthead and Letterhead</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Approval Code field shows the integrated-billing approval code</t>
+          <t>No status pill appears in the masthead on any document</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Integrated billing is not exercised on this environment. Every one of the 100 work orders reachable at Staging Heavy Duty - 9919 was read live and NOT ONE carries an ibs_approval_code - the field is null on all of them - so no document exists on which the Approval Code field could be shown. Some work orders do carry a customer IBS account number (company_ibs, for example 783799 and 783739), which shows the customers are set up for integrated billing, but no approval code has ever been issued against a work order here.</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Both clauses - that the Approval Code shows in its own field labeled exactly 'Approval Code', and that it is no longer shown under the 'Authorizer' label. To finish it: get a work order through the Interstate Billing Service approval flow so it is issued a real approval code (Administration &gt; IBS holds the integration settings, and the customer record carries an IBS field), then open that work order's document and check the Approval Code appears in its own labelled field and NOT under Authorizer.</t>
-        </is>
-      </c>
+          <t>No status label or pill anywhere in the masthead of either document (scanned the masthead band for PAID / PAID IN FULL / DRAFT / VOID / VOIDED / UNPAID / OVERDUE - zero hits on both).</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>C44951</t>
+          <t>C44905</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44951</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44905</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Paid Banner, Payments and Balance</t>
+          <t>Masthead and Letterhead</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Paid banner appears only on portal-generated Invoice PDFs, before all content</t>
+          <t>No money figure in the masthead; headline figure is the boxed total</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Clause 3 IS verified, and it is the half that can be checked from the shop app: no shop-app-generated PDF carries the banner. Confirmed across every document produced this pass - unpaid, partially paid, fully paid, deposit-paid, credit-applied and reversed - with three shop-recorded payments, an applied credit and an applied deposit between them. Not one carries a banner. The paid banner exists only on a PDF generated by the CUSTOMER PORTAL (S8-R8), which is a separate application from the shop app. It could not be reached from here: the four obvious hosts (portal./customer./pay./my.staging.shopview.com) do not resolve, and the shop-app bundle contains no portal URL at all - only the permission flags customerPortal, customerPortalPageAccess and userHasCustomerPortalAccess. There is also no portal-processed payment anywhere on the test customer: every payment ever recorded against account 4 Star Truck Repair carries the code CASH, VISA or APPLIED CREDIT, never SHOPPAY. The ShopPay and CustomerPortal feature flags ARE enabled on this organisation, so the feature exists - it simply is not reachable from the shop app.</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Clauses 1, 2, 4 and 5 - the banner's position before the masthead, its listing only portal-processed payments, the PAID IN FULL / PARTIALLY PAID pill and the batch title wording. To finish it: get the customer-portal URL for staging and a portal login for a customer contact of 4 Star Truck Repair, then pay an invoice through ShopPay in the portal and download the invoice PDF from there. The banner should then be on that PDF, before the masthead.</t>
-        </is>
-      </c>
+          <t>No monetary amount in any of the three mastheads (checked by y-coordinate over the masthead band, not by text order). Estimate's boxed headline reads 'ESTIMATED TOTAL'; Invoice's reads 'BALANCE'; the Credit Invoice has NO boxed headline and its masthead carries only 'Credit: CM-4347' and 'Issue date: Sep 7, 2026'.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>C44952</t>
+          <t>C44906</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44952</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44906</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Paid Banner, Payments and Balance</t>
+          <t>Masthead and Letterhead</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Each banner payment shows its labeled fields and conditional fees/marker</t>
+          <t>Masthead date labels read correctly for each document type</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Nothing in this case can be produced from the shop app: every field it names ('Date / Time', 'Paid By', 'Method', 'Invoice Amount', 'Total Charged', 'Convenience Fee', 'Late Fee', 'Remaining Balance', 'Payment X of Y - Batch') exists only inside the paid banner. The paid banner exists only on a PDF generated by the CUSTOMER PORTAL (S8-R8), which is a separate application from the shop app. It could not be reached from here: the four obvious hosts (portal./customer./pay./my.staging.shopview.com) do not resolve, and the shop-app bundle contains no portal URL at all - only the permission flags customerPortal, customerPortalPageAccess and userHasCustomerPortalAccess. There is also no portal-processed payment anywhere on the test customer: every payment ever recorded against account 4 Star Truck Repair carries the code CASH, VISA or APPLIED CREDIT, never SHOPPAY. The ShopPay and CustomerPortal feature flags ARE enabled on this organisation, so the feature exists - it simply is not reachable from the shop app.</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>All six clauses. To finish it: get the customer-portal URL for staging and a portal login for a customer contact of 4 Star Truck Repair, then pay an invoice through ShopPay in the portal and download the invoice PDF from there. The banner should then be on that PDF, before the masthead.</t>
-        </is>
-      </c>
+          <t>All four document types rendered and read on 2026-09-07. (1) Estimate EST-S2-32136: 'Estimate date: Sep 7, 2026' and no due-date line anywhere. (2) Unpaid Invoice INV-S2-32136: 'Invoice date: Sep 7, 2026' and 'Due date: Sep 14, 2026'. (3) Fully paid Invoice INV-S2-32136 after two payments: 'Invoice date: Sep 7, 2026' and 'Paid date: Sep 6, 2026' - Paid date replacing Due date, re-confirmed on the deposit-paid INV-S2-32217 which reads 'Paid date: Sep 1, 2026'. (4) Credit CM-4347: 'Issue date: Sep 7, 2026'. (5) Every date is in the fixed 'Sep 7, 2026' form the clause illustrates as 'Jan 5, 2026'.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>C44963</t>
+          <t>C44908</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44963</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44908</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Estimate and Invoice Specifics</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Invoice with no due date shows no Due date line; paid swap still applies</t>
+          <t>Bill To block shows the customer name and address</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Cannot be produced on staging as configured: every customer account in this organisation carries a credit term (4 Star Truck Repair is 'Net 7'), and the invoice derives its due date from that term, so an invoice with no due date could not be created through the API or the invoice-create path.</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>To finish it: clear the customer's payment terms (Customers &gt; the customer &gt; Terms) so the term is blank, then invoice a work order for that customer and read the masthead - expect 'Invoice date' with no 'Due date' line, then make it fully paid and expect 'Paid date'.</t>
-        </is>
-      </c>
+          <t>Block labeled exactly 'BILL TO' shows the company name '4 Star Truck Repair', street '6263 Elizabeth Causeway Apt. 973' and 'Raystad, British Columbia V4M 8Y2' (city, province, postal).</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>C45175</t>
+          <t>C44909</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45175</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44909</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Paid Banner, Payments and Balance</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Paid banner pill and title wording follow the paid state and the batch rule</t>
+          <t>Remit Payment To shows when a payee is configured (both mechanisms)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Nothing in this case can be produced from the shop app: the pill and the title are parts of the paid banner. The paid banner exists only on a PDF generated by the CUSTOMER PORTAL (S8-R8), which is a separate application from the shop app. It could not be reached from here: the four obvious hosts (portal./customer./pay./my.staging.shopview.com) do not resolve, and the shop-app bundle contains no portal URL at all - only the permission flags customerPortal, customerPortalPageAccess and userHasCustomerPortalAccess. There is also no portal-processed payment anywhere on the test customer: every payment ever recorded against account 4 Star Truck Repair carries the code CASH, VISA or APPLIED CREDIT, never SHOPPAY. The ShopPay and CustomerPortal feature flags ARE enabled on this organisation, so the feature exists - it simply is not reachable from the shop app.</t>
+          <t>Produced from an existing record whose location IS configured with an integrated-billing payee: work order S2-16541. Clause 1 - the block is labelled exactly 'REMIT PAYMENT TO' and holds the payee address ('Foothills Group Inc c/o Interstate Billing Service', 'C/O T04220C PO Box 4220, STN A', 'Toronto, Ontario M5W 3B9', phone). Clause 3 - it renders on both the Estimate (EST) and the Invoice (INV-S2-16541) for that record, and on none of the nine Credit documents rendered this pass.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>All three clauses. To finish it: get the customer-portal URL for staging and a portal login for a customer contact of 4 Star Truck Repair, then pay an invoice through ShopPay in the portal and download the invoice PDF from there. The banner should then be on that PDF, before the masthead.</t>
+          <t>Clause 2's second mechanism - the LOCATION's own remit-to setting, as distinct from the shop's integrated-billing remit-to - was not separately exercised. The payee here resolves through integrated billing (Interstate Billing Service). Earlier recorded as not exercised because all three workplaces on the default customer carry remit_to pointing at themselves. The condition does exist elsewhere in the estate.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>C45178</t>
+          <t>C44910</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45178</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44910</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Estimate and Invoice Specifics</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>A zero-total invoice with nothing applied is not treated as fully paid</t>
+          <t>Bill To spans full width when Remit Payment To is absent</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Cannot be produced: an invoice with a $0.00 total needs a work order whose lines total zero, and every canned line available at this location carries a price. A zero-priced line could not be created through the line-create path.</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>To finish it: build a work order with one line priced $0.00 (or discount the line to zero without applying a payment), invoice it, and read the masthead - expect 'Due date' (or no due-date line), never 'Paid date', because fully paid needs Balance $0.00 AND at least one applied row.</t>
-        </is>
-      </c>
+          <t>Clause 1 - with no Remit block, Bill To measures x0=60.0 to x1=535.3, 475.3pt, the full content width (INV-S2-32136). Clause 2 - with a payee configured (INV-S2-16541), Bill To starts at x0=60.0 and Remit Payment To at x0=308.5 inside the same 60.0-535.3 addresses row: the two sit side by side, each about half width. Clause 3 - on the Credit Invoice the Credit To block measures the same full 475.3pt (CM-4354).</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>C45190</t>
+          <t>C44911</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45190</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44911</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Cross-Cutting and Regression</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Customer card still works on work order, imported work order and part sale</t>
+          <t>Remit Payment To is hidden when no payee is configured</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Two of the three record types verified, both correct. WORK ORDER S2-32136: the customer card renders in full - '4 Star Truck Repair / Contact Savannah Tran / Phone 898-021-4480 / Authorizer Savannah Tran / Phone 898-021-4480' - and the Authorizer row carries a working dropdown control. PART SALE P2-1931: the same card renders with the same fields, and the Authorizer row is present with its dropdown, which is what clause 2 requires for a parts sale. No layout break on either.</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>The IMPORTED WORK ORDER half of both clauses. There is no imported work order anywhere in this organisation: GET /api/work-orders-imported returns an empty list at Staging Heavy Duty - 9919, and the same query filtered by the customer returns none. So the card could not be seen on an imported work order, and the rule that the Authorizer row must be ABSENT there could not be exercised. To finish it: import a work order (or ask for one to be seeded), open it, and check two things - the customer card renders without a layout break, and the Authorizer row is NOT shown on it. Everything else in this case has already passed.</t>
-        </is>
-      </c>
+          <t>Both clauses observed. No 'Remit Payment To' block on either document, and the shop's own address appears ONLY in the masthead - it is not reprinted as a fallback remit-to. Confirmed from the record: workplace remitToAddress = None.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>C45275</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45275</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Authorizer Entry (Work Order)</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Changing the customer clears the Authorizer; changing only the contact does not</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>The case cannot be scored: its Steps field and its Expected Results field are both EMPTY in TestRail. Only the preconditions and the title are written, so there is nothing for a tester to follow and no documented expectation to judge against.</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>The behaviour its title describes was exercised anyway and holds: with the Authorizer set to Savannah Tran on S-32222, changing only the CONTACT (to ZZAUTOTEST NewApprover) left the Authorizer as Savannah Tran; changing the CUSTOMER (4 Star Truck Repair -&gt; 7 Star Truck Repair) cleared it to None. Recorded as an observation, not a verdict. The empty case needs Steps and Expected Results before a tester can run it - reported to the QA lead, not edited (this lane does not author cases).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G107"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>C-ID</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>TestRail link</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Case title</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>What was observed</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>What still needs doing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>C44901</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44901</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Masthead and Letterhead</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Masthead shows the shop location's full identity details</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>All five identity values match the shop record byte-for-byte: name 'Staging Heavy Duty - 9919', '9919 Shepard Road SE', 'Calgary, Alberta', 'T2C 4M5', '(403) 523 - 0488' (GET /api/workplaces).</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>C44903</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44903</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Masthead and Letterhead</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Document label names the type before the number on each document</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>All three document labels now observed: 'Estimate: EST-S2-32136', 'Invoice: INV-S2-32136' and 'Credit: CM-4347'. In each the type word precedes the number and the number carries its type prefix (EST- / INV- / CM-).</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>The Invoices LIST renders the credit as 'CM2-4347', but the DOCUMENT reads 'CM-4347' - the document is what this case asserts, and it is correct.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>C44904</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44904</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Masthead and Letterhead</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>No status pill appears in the masthead on any document</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>No status label or pill anywhere in the masthead of either document (scanned the masthead band for PAID / PAID IN FULL / DRAFT / VOID / VOIDED / UNPAID / OVERDUE - zero hits on both).</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>C44905</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44905</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Masthead and Letterhead</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>No money figure in the masthead; headline figure is the boxed total</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>No monetary amount in any of the three mastheads (checked by y-coordinate over the masthead band, not by text order). Estimate's boxed headline reads 'ESTIMATED TOTAL'; Invoice's reads 'BALANCE'; the Credit Invoice has NO boxed headline and its masthead carries only 'Credit: CM-4347' and 'Issue date: Sep 7, 2026'.</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>C44906</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44906</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Masthead and Letterhead</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Masthead date labels read correctly for each document type</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>All four document types rendered and read on 2026-09-07. (1) Estimate EST-S2-32136: 'Estimate date: Sep 7, 2026' and no due-date line anywhere. (2) Unpaid Invoice INV-S2-32136: 'Invoice date: Sep 7, 2026' and 'Due date: Sep 14, 2026'. (3) Fully paid Invoice INV-S2-32136 after two payments: 'Invoice date: Sep 7, 2026' and 'Paid date: Sep 6, 2026' - Paid date replacing Due date, re-confirmed on the deposit-paid INV-S2-32217 which reads 'Paid date: Sep 1, 2026'. (4) Credit CM-4347: 'Issue date: Sep 7, 2026'. (5) Every date is in the fixed 'Sep 7, 2026' form the clause illustrates as 'Jan 5, 2026'.</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>C44908</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44908</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Addresses</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Bill To block shows the customer name and address</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Block labeled exactly 'BILL TO' shows the company name '4 Star Truck Repair', street '6263 Elizabeth Causeway Apt. 973' and 'Raystad, British Columbia V4M 8Y2' (city, province, postal).</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>C44909</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44909</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Addresses</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Remit Payment To shows when a payee is configured (both mechanisms)</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Produced from an existing record whose location IS configured with an integrated-billing payee: work order S2-16541. Clause 1 - the block is labelled exactly 'REMIT PAYMENT TO' and holds the payee address ('Foothills Group Inc c/o Interstate Billing Service', 'C/O T04220C PO Box 4220, STN A', 'Toronto, Ontario M5W 3B9', phone). Clause 3 - it renders on both the Estimate (EST) and the Invoice (INV-S2-16541) for that record, and on none of the nine Credit documents rendered this pass.</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Clause 2's second mechanism - the LOCATION's own remit-to setting, as distinct from the shop's integrated-billing remit-to - was not separately exercised. The payee here resolves through integrated billing (Interstate Billing Service). Earlier recorded as not exercised because all three workplaces on the default customer carry remit_to pointing at themselves. The condition does exist elsewhere in the estate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>C44910</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44910</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Addresses</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Bill To spans full width when Remit Payment To is absent</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Clause 1 - with no Remit block, Bill To measures x0=60.0 to x1=535.3, 475.3pt, the full content width (INV-S2-32136). Clause 2 - with a payee configured (INV-S2-16541), Bill To starts at x0=60.0 and Remit Payment To at x0=308.5 inside the same 60.0-535.3 addresses row: the two sit side by side, each about half width. Clause 3 - on the Credit Invoice the Credit To block measures the same full 475.3pt (CM-4354).</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>C44911</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44911</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Addresses</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Remit Payment To is hidden when no payee is configured</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Both clauses observed. No 'Remit Payment To' block on either document, and the shop's own address appears ONLY in the masthead - it is not reprinted as a fallback remit-to. Confirmed from the record: workplace remitToAddress = None.</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
           <t>C44912</t>
         </is>
       </c>
@@ -1623,12 +1475,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Labels read exactly and carry NO punctuation: 'Customer PO 9989', 'Authorizer Savannah Tran', 'Terms Net 7'. The three present appear in the specified relative order (Customer PO -&gt; Authorizer -&gt; Terms).</t>
+          <t>Clause 2 - no label carries punctuation: 'Customer PO 9989', 'Authorizer Savannah Tran', 'Terms Net 7', no colons. Clause 3 - the labels read exactly as the rule lists them. Clause 1 - the three fields present appear in the specified relative order, Customer PO then Authorizer then Terms.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Work Order and Approval Code were not present, so the full five-field order was not exercised - both are correctly hidden by their own rules on this record (and see SV-9770 on Work Order).</t>
+          <t>The full five-field order could not be observed. The 'Work Order' field, which leads the fixed order, is absent from the build, and the 'Approval Code' field has never been populated on this environment (C44916). So the order was verified across three of the five, not all five. The missing Work Order field is the SV-9642 defect recorded under C44917, not a separate fault of this case. Once that is fixed, re-run this case to confirm the Work Order field takes first position in the row.</t>
         </is>
       </c>
     </row>
@@ -1705,12 +1557,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>C44917</t>
+          <t>C44918</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44917</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44918</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1720,7 +1572,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Work Order field hides when it equals the document number's trailing digits</t>
+          <t>Customer PO, Authorizer and Approval Code each hide when empty</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1730,34 +1582,34 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 holds on the build. Work order S-32136 (the value GET /api/work-orders/view returns; the Work Orders grid shows it as S2-32136) against documents EST-S2-32136 and INV-S2-32136: the unbroken trailing digits are '32136' on both sides, they are equal, and the Work Order field is correctly absent from the order-reference row on both documents.</t>
+          <t>Read on INV-S2-32217, a work order deliberately created with no customer PO and no authorizer. Clause 1: no 'Customer PO' label and no empty value area - the field is absent entirely. Clause 2: no 'Authorizer' label and no empty value area. Clause 4: 'Terms Net 7' still shows, the always-show exception. The contrast document INV-S2-32136, which has both, prints 'Customer PO 9989' and 'Authorizer Savannah Tran', so the fields do render when populated - the absence above is the hide rule firing, not a missing feature.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 - the field SHOWING when the two differ. It could not be produced: a document number is derived from the work order number, so on an ordinary document the trailing digits always match and the hide condition is always true. Clause 2's unproducibility is the substance of the open question already raised as SV-9770 (a Task carrying the Clarification_needed label, awaiting Chris Ward). Nothing further to raise here - the build follows the rule as written.</t>
+          <t>Clause 3 (Approval Code hidden when empty) is satisfied on the page - no Approval Code label appears - but it is a weak observation: integrated billing is not configured on this organisation, so the field has never been seen populated and its hide rule has not been exercised against a real value.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>C44918</t>
+          <t>C44919</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44918</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44919</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Order Reference Fields</t>
+          <t>Authorizer Entry (Work Order)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Customer PO, Authorizer and Approval Code each hide when empty</t>
+          <t>Authorizer is selected in the work order customer contact card</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1767,24 +1619,24 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Read on INV-S2-32217, a work order deliberately created with no customer PO and no authorizer. Clause 1: no 'Customer PO' label and no empty value area - the field is absent entirely. Clause 2: no 'Authorizer' label and no empty value area. Clause 4: 'Terms Net 7' still shows, the always-show exception. The contrast document INV-S2-32136, which has both, prints 'Customer PO 9989' and 'Authorizer Savannah Tran', so the fields do render when populated - the absence above is the hide rule firing, not a missing feature.</t>
+          <t>Driven in the browser on work order S-32222 (and corroborated on S2-15501). Clause 1 - an 'Authorizer' row appears in the customer contact card directly below the Contact name and its Phone, in the same label-above-value style. Clause 2 - opening it lists only the customer's contacts flagged 'Approves Work': the list showed 'No authorizer' and 'Savannah Tran'; a contact of the SAME customer created without the flag (ZZAUTOTEST NonApprover) was NOT offered. Clause 3 - no other contact is offered, and no free-typed name is possible: the control's input carries readonly and aria-autocomplete="none" (data-test-id=select_authorizer). Clause 4 - select_authorizer is the only authorizer control in the app; the parts sale carries its own equivalent under S13-R6, which is the documented exception rather than a second place on the work order.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Clause 3 (Approval Code hidden when empty) is satisfied on the page - no Approval Code label appears - but it is a weak observation: integrated billing is not configured on this organisation, so the field has never been seen populated and its hide rule has not been exercised against a real value.</t>
+          <t>Route recorded: Work Orders -&gt; the row -&gt; /workorders/{id}/lines, customer contact card on the left.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>C44919</t>
+          <t>C44920</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44919</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44920</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1794,7 +1646,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Authorizer is selected in the work order customer contact card</t>
+          <t>Authorizer is optional and can be cleared with 'No authorizer'</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1804,24 +1656,20 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Driven in the browser on work order S-32222 (and corroborated on S2-15501). Clause 1 - an 'Authorizer' row appears in the customer contact card directly below the Contact name and its Phone, in the same label-above-value style. Clause 2 - opening it lists only the customer's contacts flagged 'Approves Work': the list showed 'No authorizer' and 'Savannah Tran'; a contact of the SAME customer created without the flag (ZZAUTOTEST NonApprover) was NOT offered. Clause 3 - no other contact is offered, and no free-typed name is possible: the control's input carries readonly and aria-autocomplete="none" (data-test-id=select_authorizer). Clause 4 - select_authorizer is the only authorizer control in the app; the parts sale carries its own equivalent under S13-R6, which is the documented exception rather than a second place on the work order.</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Route recorded: Work Orders -&gt; the row -&gt; /workorders/{id}/lines, customer contact card on the left.</t>
-        </is>
-      </c>
+          <t>Clause 1 - a newly created work order shows 'Authorizer  None'; the field is not required and nothing blocks saving. Clause 2 - the list's first entry is 'No authorizer'. Clause 3 - with 'Savannah Tran' selected, choosing 'No authorizer' returned the row to 'None' and cleared the stored value (a live re-read shows authorizer_full_name null).</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>C44920</t>
+          <t>C44921</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44920</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44921</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1831,7 +1679,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Authorizer is optional and can be cleared with 'No authorizer'</t>
+          <t>Authorizer's phone shows below the name when the contact has one</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1841,7 +1689,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - a newly created work order shows 'Authorizer  None'; the field is not required and nothing blocks saving. Clause 2 - the list's first entry is 'No authorizer'. Clause 3 - with 'Savannah Tran' selected, choosing 'No authorizer' returned the row to 'None' and cleared the stored value (a live re-read shows authorizer_full_name null).</t>
+          <t>Clause 1 - with 'Savannah Tran' selected (contact telephone 898-021-4480), the card shows 'Phone  898-021-4480' directly below the authorizer's name, in the same treatment as the Contact's phone. Clause 2 - a purpose-made approver with no telephone on the contact record (ZZAUTOTEST NoPhoneApprover) shows the name with NO phone row beneath it.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr"/>
@@ -1849,12 +1697,12 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>C44921</t>
+          <t>C44922</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44921</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44922</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1864,7 +1712,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Authorizer's phone shows below the name when the contact has one</t>
+          <t>Authorizer is locked once the work order is invoiced</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1874,7 +1722,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - with 'Savannah Tran' selected (contact telephone 898-021-4480), the card shows 'Phone  898-021-4480' directly below the authorizer's name, in the same treatment as the Contact's phone. Clause 2 - a purpose-made approver with no telephone on the contact record (ZZAUTOTEST NoPhoneApprover) shows the name with NO phone row beneath it.</t>
+          <t>Clause 1 - on invoiced work order S2-32221 the Authorizer control renders as static text: no input element, no role="combobox", and a click times out because nothing is clickable. Clause 2 - before invoicing the same control on S-32222 carries a readonly combobox input that opens the list. Clause 3 - reversing that invoice re-enabled the row within the same session: after a reload the input and combobox were back and the list opened with all four options. The server agrees - the same change is HTTP 409 while invoiced and HTTP 200 after the reversal.</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr"/>
@@ -1882,12 +1730,12 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>C44922</t>
+          <t>C44923</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44922</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44923</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1897,7 +1745,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Authorizer is locked once the work order is invoiced</t>
+          <t>A new 'Approves Work' contact becomes selectable immediately</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1907,7 +1755,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - on invoiced work order S2-32221 the Authorizer control renders as static text: no input element, no role="combobox", and a click times out because nothing is clickable. Clause 2 - before invoicing the same control on S-32222 carries a readonly combobox input that opens the list. Clause 3 - reversing that invoice re-enabled the row within the same session: after a reload the input and combobox were back and the list opened with all four options. The server agrees - the same change is HTTP 409 while invoiced and HTTP 200 after the reversal.</t>
+          <t>With the work order open and the Authorizer list already inspected (it held 'No authorizer' and 'Savannah Tran'), a new contact flagged 'Approves Work' was created against the same customer. Re-opening the list on the SAME page, with no reload and no re-save of the work order, showed 'No authorizer', 'ZZAUTOTEST NewApprover' and 'Savannah Tran' - the new contact is selectable immediately.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
@@ -1915,22 +1763,22 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>C44923</t>
+          <t>C44924</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44923</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44924</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Authorizer Entry (Work Order)</t>
+          <t>Asset Section</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>A new 'Approves Work' contact becomes selectable immediately</t>
+          <t>Asset section shows Asset name and VIN / Serial when present</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1940,20 +1788,24 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>With the work order open and the Authorizer list already inspected (it held 'No authorizer' and 'Savannah Tran'), a new contact flagged 'Approves Work' was created against the same customer. Re-opening the list on the SAME page, with no reload and no re-save of the work order, showed 'No authorizer', 'ZZAUTOTEST NewApprover' and 'Savannah Tran' - the new contact is selectable immediately.</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr"/>
+          <t>Clauses 1, 2 and 4 observed: 'ASSET  2011 Hyundai Santa Fe' and 'VIN / SERIAL  PV1T2SK1DNUUK7YDE' - the asset has a VIN and the VIN is what prints.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Clause 3 (serial shown when there is no VIN) not exercised.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>C44924</t>
+          <t>C44925</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44924</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44925</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1963,7 +1815,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Asset section shows Asset name and VIN / Serial when present</t>
+          <t>Asset section can show Unit, Plate, Mileage and Eng Hrs</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1973,24 +1825,20 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Clauses 1, 2 and 4 observed: 'ASSET  2011 Hyundai Santa Fe' and 'VIN / SERIAL  PV1T2SK1DNUUK7YDE' - the asset has a VIN and the VIN is what prints.</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Clause 3 (serial shown when there is no VIN) not exercised.</t>
-        </is>
-      </c>
+          <t>All four fields present with values: 'UNIT 665', 'PLATE ZZP-6028', 'MILEAGE 45', 'ENG HRS 9,987', each labeled exactly as specified.</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>C44925</t>
+          <t>C44927</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44925</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44927</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2000,7 +1848,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Asset section can show Unit, Plate, Mileage and Eng Hrs</t>
+          <t>VIN / Serial hides when the asset has neither; Asset name still shows</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -2010,20 +1858,24 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>All four fields present with values: 'UNIT 665', 'PLATE ZZP-6028', 'MILEAGE 45', 'ENG HRS 9,987', each labeled exactly as specified.</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr"/>
+          <t>Seeded an asset with no VIN and no serial number (vehicle created with a year only) and invoiced it as INV-S2-32225. The 'VIN / SERIAL' field is absent from the asset band entirely - no label, no empty value. The asset name still shows, reading '2019'. The contrast is the reference document INV-S2-32136, whose asset does have a VIN and prints 'VIN / SERIAL  PV1T2SK1DNUUK7YDE', so the field renders when there is something to render.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>S4-N2's 'Unknown' variant (a VIN or serial literally reading 'Unknown' in any casing counts as none) was not exercised - only the genuinely-empty case.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>C44927</t>
+          <t>C44928</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44927</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44928</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2033,7 +1885,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>VIN / Serial hides when the asset has neither; Asset name still shows</t>
+          <t>Asset section shows whenever the work order has an asset (parts sales too)</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -2043,34 +1895,34 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Seeded an asset with no VIN and no serial number (vehicle created with a year only) and invoiced it as INV-S2-32225. The 'VIN / SERIAL' field is absent from the asset band entirely - no label, no empty value. The asset name still shows, reading '2019'. The contrast is the reference document INV-S2-32136, whose asset does have a VIN and prints 'VIN / SERIAL  PV1T2SK1DNUUK7YDE', so the field renders when there is something to render.</t>
+          <t>Both clauses, on part sales specifically. Clause 1: part sale P2-1932, created with the Santa Fe attached, renders the full asset band exactly as a service work order does - 'ASSET 2011 Hyundai Santa Fe / UNIT 665 / PLATE ZZP-6028 / MILEAGE 45 / ENG HRS 0 / VIN / SERIAL PV1T2SK1DNUUK7YDE'. Clause 2: part sale P2-1931, which has no asset, hides the section entirely. Same document type, same shop, the only difference being whether an asset is attached.</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>S4-N2's 'Unknown' variant (a VIN or serial literally reading 'Unknown' in any casing counts as none) was not exercised - only the genuinely-empty case.</t>
+          <t>The 'ENG HRS 0' in the band above is the SV-9680 zero-instead-of-hidden problem recorded under C44926, not a fault of this case.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>C44928</t>
+          <t>C44929</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44928</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44929</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Asset Section</t>
+          <t>Work Section</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Asset section shows whenever the work order has an asset (parts sales too)</t>
+          <t>Work heading is 'Work Summary' on Estimate and 'Work Performed' on Invoice</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2080,24 +1932,20 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Both clauses, on part sales specifically. Clause 1: part sale P2-1932, created with the Santa Fe attached, renders the full asset band exactly as a service work order does - 'ASSET 2011 Hyundai Santa Fe / UNIT 665 / PLATE ZZP-6028 / MILEAGE 45 / ENG HRS 0 / VIN / SERIAL PV1T2SK1DNUUK7YDE'. Clause 2: part sale P2-1931, which has no asset, hides the section entirely. Same document type, same shop, the only difference being whether an asset is attached.</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>The 'ENG HRS 0' in the band above is the SV-9680 zero-instead-of-hidden problem recorded under C44926, not a fault of this case.</t>
-        </is>
-      </c>
+          <t>Estimate heading reads 'WORK SUMMARY'; Invoice heading reads 'WORK PERFORMED'. Both captured from the build; the difference is exactly as specified.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>C44929</t>
+          <t>C44930</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44929</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44930</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2107,7 +1955,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Work heading is 'Work Summary' on Estimate and 'Work Performed' on Invoice</t>
+          <t>Work line numbers are sequential and zero-padded to two digits</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2117,20 +1965,24 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Estimate heading reads 'WORK SUMMARY'; Invoice heading reads 'WORK PERFORMED'. Both captured from the build; the difference is exactly as specified.</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr"/>
+          <t>Line numbers render 01, 02, 03 - sequential, no gaps, zero-padded to two digits, at 13.5pt (=18px).</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>The 100+ line three-digit case is C45173's job and was not exercised here.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>C44930</t>
+          <t>C44931</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44930</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44931</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2140,7 +1992,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Work line numbers are sequential and zero-padded to two digits</t>
+          <t>Each work line shows name, and description and scope-of-work note when present</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -2150,24 +2002,24 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Line numbers render 01, 02, 03 - sequential, no gaps, zero-padded to two digits, at 13.5pt (=18px).</t>
+          <t>Line 01 shows name 'ABCD', description 'EFGH' inline in smaller muted text (9.0pt = 12px), and a SCOPE OF WORK note 'Eeee' below. Lines 02 and 03 the same shape.</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>The 100+ line three-digit case is C45173's job and was not exercised here.</t>
+          <t>Clause 4 (a line with neither description nor scope note) not exercised - all three lines have both.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>C44931</t>
+          <t>C44932</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44931</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44932</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2177,7 +2029,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Each work line shows name, and description and scope-of-work note when present</t>
+          <t>Labor and Parts entries are labeled exactly 'Labor' and 'Parts'</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -2187,24 +2039,20 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Line 01 shows name 'ABCD', description 'EFGH' inline in smaller muted text (9.0pt = 12px), and a SCOPE OF WORK note 'Eeee' below. Lines 02 and 03 the same shape.</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Clause 4 (a line with neither description nor scope note) not exercised - all three lines have both.</t>
-        </is>
-      </c>
+          <t>Labor entries are labeled 'LABOR' and parts entries 'PARTS' (uppercase is the document's text-transform; capitalisation alone is not a divergence).</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>C44932</t>
+          <t>C44933</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44932</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44933</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2214,7 +2062,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Labor and Parts entries are labeled exactly 'Labor' and 'Parts'</t>
+          <t>Invoice Details settings show or hide the per-entry figures</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -2224,20 +2072,24 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Labor entries are labeled 'LABOR' and parts entries 'PARTS' (uppercase is the document's text-transform; capitalisation alone is not a divergence).</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr"/>
+          <t>Every one of the seven per-entry settings A/B-tested on the Finance tab of WO S2-32136, line 02 (which carries one labor entry and two parts entries), turning each off and back on and reading the document each time. Clause 1, all on: the labor entry shows hours, rate and amount; each parts entry shows the part number, the description, the quantity, the rate and the amount. Clause 2, each off hides its own figure and nothing else - 'Labor rate' removes the $149.95 rate, 'Labor hours' removes the quantity, 'Part quantity' removes the part quantity, 'Part number' removes the 'N68SL-356 - ' prefix leaving the description, 'Part description' removes the description leaving 'N68SL-356', and 'Part price' removes both the part rate and the part amount. Clause 3: 'Labor price' off ALSO removes the line footer's 'Labor' figure, leaving 'Parts $48.31  Line total $198.26'; and 'Part price' off likewise removes the footer's 'Parts' figure, leaving 'Labor $149.95  Line total $198.26'.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>The settings live behind the gear icon on the Finance tab and their test ids are not the camel-case of their labels - 'Labor price' is toggle_setting_laborCost and 'Part price' is toggle_setting_partCost.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>C44933</t>
+          <t>C44934</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44933</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44934</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2247,7 +2099,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Invoice Details settings show or hide the per-entry figures</t>
+          <t>Line-level fee shows as a plain amount; discount shows in parentheses</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -2257,24 +2109,20 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Every one of the seven per-entry settings A/B-tested on the Finance tab of WO S2-32136, line 02 (which carries one labor entry and two parts entries), turning each off and back on and reading the document each time. Clause 1, all on: the labor entry shows hours, rate and amount; each parts entry shows the part number, the description, the quantity, the rate and the amount. Clause 2, each off hides its own figure and nothing else - 'Labor rate' removes the $149.95 rate, 'Labor hours' removes the quantity, 'Part quantity' removes the part quantity, 'Part number' removes the 'N68SL-356 - ' prefix leaving the description, 'Part description' removes the description leaving 'N68SL-356', and 'Part price' removes both the part rate and the part amount. Clause 3: 'Labor price' off ALSO removes the line footer's 'Labor' figure, leaving 'Parts $48.31  Line total $198.26'; and 'Part price' off likewise removes the footer's 'Parts' figure, leaving 'Labor $149.95  Line total $198.26'.</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>The settings live behind the gear icon on the Finance tab and their test ids are not the camel-case of their labels - 'Labor price' is toggle_setting_laborCost and 'Part price' is toggle_setting_partCost.</t>
-        </is>
-      </c>
+          <t>On work order S2-32229, line 01 carries a labor-scoped fee of $20.00 and a labor-scoped discount of $5.00. The document prints them beneath the line as '↳ ZZ Labor Fee   $20.00' (a plain amount) and '↳ ZZ Labor Discount   ($5.00)' (in parentheses). Clause 3 holds literally: the parentheses are characters in the extracted text, not a colour or a font treatment - the same figure without parentheses would extract differently.</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>C44934</t>
+          <t>C44936</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44934</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44936</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2284,7 +2132,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Line-level fee shows as a plain amount; discount shows in parentheses</t>
+          <t>Empty work section shows heading; Summary divider still precedes summary</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -2294,7 +2142,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>On work order S2-32229, line 01 carries a labor-scoped fee of $20.00 and a labor-scoped discount of $5.00. The document prints them beneath the line as '↳ ZZ Labor Fee   $20.00' (a plain amount) and '↳ ZZ Labor Discount   ($5.00)' (in parentheses). Clause 3 holds literally: the parentheses are characters in the extracted text, not a colour or a font treatment - the same figure without parentheses would extract differently.</t>
+          <t>Rendered the Estimate for work order S2-32228, created with no work lines at all. The work-section heading 'WORK SUMMARY' prints with nothing beneath it, and the 'SUMMARY' divider still follows it and precedes the financial summary. Corroborated on part sale P2-1932, whose 'PARTS' heading prints empty and is likewise followed by the SUMMARY divider.</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr"/>
@@ -2302,22 +2150,22 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>C44936</t>
+          <t>C44937</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44936</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44937</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Work Section</t>
+          <t>Declined Work</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Empty work section shows heading; Summary divider still precedes summary</t>
+          <t>Declined Work shows in its own section with names and descriptions only</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -2327,7 +2175,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Rendered the Estimate for work order S2-32228, created with no work lines at all. The work-section heading 'WORK SUMMARY' prints with nothing beneath it, and the 'SUMMARY' divider still follows it and precedes the financial summary. Corroborated on part sale P2-1932, whose 'PARTS' heading prints empty and is likewise followed by the SUMMARY divider.</t>
+          <t>With declined work shown, a section headed exactly 'DECLINED WORK' renders separately from the work section. The declined line shows its name ('What are you doing 4th line (Decline)') and its description ('Whya re you doing 4th line (Decline)'). Clause 3 holds: NO scope-of-work note appears under it - the next element is the SUMMARY divider.</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
@@ -2335,12 +2183,12 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>C44937</t>
+          <t>C44938</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44937</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44938</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2350,7 +2198,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Declined Work shows in its own section with names and descriptions only</t>
+          <t>Declined lines show no prices, no line numbers, and no status pill</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2360,7 +2208,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>With declined work shown, a section headed exactly 'DECLINED WORK' renders separately from the work section. The declined line shows its name ('What are you doing 4th line (Decline)') and its description ('Whya re you doing 4th line (Decline)'). Clause 3 holds: NO scope-of-work note appears under it - the next element is the SUMMARY divider.</t>
+          <t>All four clauses. The declined line carries no price, no labor or parts figure, and no line number (the numbered lines stop at 03). No status pill. And it enters no total: the summary figures are IDENTICAL between the plain and declined captures - $711.09 / $35.57 / $746.66 in both.</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
@@ -2368,12 +2216,12 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>C44938</t>
+          <t>C44939</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44938</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44939</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2383,7 +2231,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Declined lines show no prices, no line numbers, and no status pill</t>
+          <t>Declined Work section hidden when nothing declined or option off</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -2393,30 +2241,34 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>All four clauses. The declined line carries no price, no labor or parts figure, and no line number (the numbered lines stop at 03). No status pill. And it enters no total: the summary figures are IDENTICAL between the plain and declined captures - $711.09 / $35.57 / $746.66 in both.</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr"/>
+          <t>Clause 2 observed directly: the same work order rendered WITHOUT the declined option shows no Declined Work section at all, while WITH it the section appears. So the option genuinely governs visibility.</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Clause 1 (no declined lines at all) not exercised - this work order has one.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>C44939</t>
+          <t>C44940</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44939</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44940</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Declined Work</t>
+          <t>Financial Summary</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Declined Work section hidden when nothing declined or option off</t>
+          <t>'Summary' divider precedes the financial summary</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2426,24 +2278,20 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 observed directly: the same work order rendered WITHOUT the declined option shows no Declined Work section at all, while WITH it the section appears. So the option genuinely governs visibility.</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Clause 1 (no declined lines at all) not exercised - this work order has one.</t>
-        </is>
-      </c>
+          <t>A divider labeled 'SUMMARY' sits at y=220.4, immediately above the financial summary block which starts at y=247.9. Order confirmed by coordinate, not by text order.</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>C44940</t>
+          <t>C44941</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44940</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44941</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2453,7 +2301,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>'Summary' divider precedes the financial summary</t>
+          <t>Summary shows gross Labor and Parts rows, and Shop supplies when charged</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2463,7 +2311,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>A divider labeled 'SUMMARY' sits at y=220.4, immediately above the financial summary block which starts at y=247.9. Order confirmed by coordinate, not by text order.</t>
+          <t>Rows labeled 'Labor' ($599.80), 'Parts' ($48.31) and 'Shop supplies (10.5% of labor)' ($62.98) all present. Labor reconciles to the three line labor amounts (299.90+149.95+149.95) and Parts to the two part amounts (8.31+40.00), i.e. gross.</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr"/>
@@ -2471,12 +2319,12 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>C44941</t>
+          <t>C44942</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44941</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44942</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2486,7 +2334,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Summary shows gross Labor and Parts rows, and Shop supplies when charged</t>
+          <t>Shop supplies shows its percentage when the location setting is enabled</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -2496,20 +2344,24 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Rows labeled 'Labor' ($599.80), 'Parts' ($48.31) and 'Shop supplies (10.5% of labor)' ($62.98) all present. Labor reconciles to the three line labor amounts (299.90+149.95+149.95) and Parts to the two part amounts (8.31+40.00), i.e. gross.</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr"/>
+          <t>Clause 1 observed: the percentage IS shown alongside the amount - 'Shop supplies (10.5% of labor)  $62.98'. Confirmed at record level too: the workplace carries shop_supplies_charge = 10.5 with shopSupplyPercentageEnabled = true, and 10.5% of labor 599.80 = 62.98 exactly.</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Clause 2 (setting off -&gt; amount alone) not exercised on my own capture.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>C44942</t>
+          <t>C44943</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44942</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44943</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -2519,7 +2371,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Shop supplies shows its percentage when the location setting is enabled</t>
+          <t>Adjustments group shows rollup Labor/Parts then each work-order-wide row</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -2529,24 +2381,24 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 observed: the percentage IS shown alongside the amount - 'Shop supplies (10.5% of labor)  $62.98'. Confirmed at record level too: the workplace carries shop_supplies_charge = 10.5 with shopSupplyPercentageEnabled = true, and 10.5% of labor 599.80 = 62.98 exactly.</t>
+          <t>All four clauses on work order S2-32229, which carries two line-level labor adjustments and two work-order-wide ones. Clause 1: the heading reads exactly 'Adjustments' and carries no amount of its own. Clause 2: the rows appear in the specified order - the 'Labor' rollup first, then each work-order-wide row in the order it was added ('ZZ WO Fee' then 'ZZ WO Discount'). Clause 3: with line-level adjustments of +$20.00 and -$5.00 the rollup shows as a plain '$15.00'; adding a further -$40.00 flips it and it then shows as '($25.00)' in parentheses - both directions observed on the same record. The 'Parts' rollup is correctly absent throughout, its total being zero. Clause 4: the work-order-wide discount shows '($100.00)' and the work-order-wide fee shows '$75.00'. The arithmetic ties out: 350.00 + 0.00 + 36.75 - 25.00 + 75.00 - 100.00 = 336.75 Subtotal, GST 5% = 16.84, Total 353.59.</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 (setting off -&gt; amount alone) not exercised on my own capture.</t>
+          <t>The line footer on this document again excludes the line's own adjustments, which is the separate defect SV-9773; the Summary figures above are all correct.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>C44943</t>
+          <t>C44944</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44943</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44944</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2556,7 +2408,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Adjustments group shows rollup Labor/Parts then each work-order-wide row</t>
+          <t>Summary shows Subtotal, one row per tax, and the grand Total</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -2566,24 +2418,20 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>All four clauses on work order S2-32229, which carries two line-level labor adjustments and two work-order-wide ones. Clause 1: the heading reads exactly 'Adjustments' and carries no amount of its own. Clause 2: the rows appear in the specified order - the 'Labor' rollup first, then each work-order-wide row in the order it was added ('ZZ WO Fee' then 'ZZ WO Discount'). Clause 3: with line-level adjustments of +$20.00 and -$5.00 the rollup shows as a plain '$15.00'; adding a further -$40.00 flips it and it then shows as '($25.00)' in parentheses - both directions observed on the same record. The 'Parts' rollup is correctly absent throughout, its total being zero. Clause 4: the work-order-wide discount shows '($100.00)' and the work-order-wide fee shows '$75.00'. The arithmetic ties out: 350.00 + 0.00 + 36.75 - 25.00 + 75.00 - 100.00 = 336.75 Subtotal, GST 5% = 16.84, Total 353.59.</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>The line footer on this document again excludes the line's own adjustments, which is the separate defect SV-9773; the Summary figures above are all correct.</t>
-        </is>
-      </c>
+          <t>All four clauses hold. 'Subtotal $711.09'; one tax row per tax, labeled with name and rate, 'GST (5%) $35.57'; grand 'Total $746.66'. The visible math reconciles: 599.80 + 48.31 + 62.98 = 711.09, and 711.09 + 35.57 = 746.66. (The tax is not a flat 5% of the subtotal because the location's salesTaxRoundingMode is 'line_by_line' - tax summed per line.)</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>C44944</t>
+          <t>C44945</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44944</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44945</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2593,7 +2441,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Summary shows Subtotal, one row per tax, and the grand Total</t>
+          <t>Adjustments heading and tax rows hide when nothing applies</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2603,30 +2451,34 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>All four clauses hold. 'Subtotal $711.09'; one tax row per tax, labeled with name and rate, 'GST (5%) $35.57'; grand 'Total $746.66'. The visible math reconciles: 599.80 + 48.31 + 62.98 = 711.09, and 711.09 + 35.57 = 746.66. (The tax is not a flat 5% of the subtotal because the location's salesTaxRoundingMode is 'line_by_line' - tax summed per line.)</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr"/>
+          <t>Clause 1 observed: no Adjustments heading appears, and there is nothing to list under it.</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Clause 2 (no tax -&gt; no tax row) not exercised - GST applies to this location.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>C44945</t>
+          <t>C44946</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44945</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44946</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Financial Summary</t>
+          <t>Paid Banner, Payments and Balance</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Adjustments heading and tax rows hide when nothing applies</t>
+          <t>Payments heading and each applied payment row show correctly</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2636,24 +2488,20 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 observed: no Adjustments heading appears, and there is nothing to list under it.</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>Clause 2 (no tax -&gt; no tax row) not exercised - GST applies to this location.</t>
-        </is>
-      </c>
+          <t>Heading reads exactly 'Payments'. Rows render as '{date} - {method}' with a literal hyphen: 'Sep 5, 2026 - Cash', 'Sep 6, 2026 - Check', 'Sep 7, 2026 - Cash', 'Sep 7, 2026 - EFT'. Amount column shows the APPLIED amount, proven by the split payment whose full amount was $397.96 but which printed $50.00 (the part applied here). Rows are date-ordered, and a fully reversed payment does not appear.</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>C44946</t>
+          <t>C44947</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44946</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44947</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2663,7 +2511,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Payments heading and each applied payment row show correctly</t>
+          <t>Payment method name resolves per rule (SHOPPAY shows 'Online')</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -2673,20 +2521,24 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Heading reads exactly 'Payments'. Rows render as '{date} - {method}' with a literal hyphen: 'Sep 5, 2026 - Cash', 'Sep 6, 2026 - Check', 'Sep 7, 2026 - Cash', 'Sep 7, 2026 - EFT'. Amount column shows the APPLIED amount, proven by the split payment whose full amount was $397.96 but which printed $50.00 (the part applied here). Rows are date-ordered, and a fully reversed payment does not appear.</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr"/>
+          <t>Clause 1 observed for three distinct configured methods: code CASH prints 'Cash', code CHEQUE prints 'Check', code EFT prints 'EFT' - in each case the shop-configured NAME from GET /api/organizations/finance/payment-methods, not the code.</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Clause 2 (an unconfigured payment code rendering with underscores turned into spaces) was not produced this pass - the API refuses an unconfigured code. Clause 3 IS now observed: a ShopPay/portal payment prints as 'Sep 7, 2026 - Online' in the Payments section of the invoice document (S-32052, which carries one CASH and one portal payment and prints 'Cash' and 'Online' side by side). Passed on the clause that could be produced; the two unproduced clauses are listed in the not_observed field rather than assumed.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>C44947</t>
+          <t>C44948</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44947</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44948</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2696,7 +2548,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Payment method name resolves per rule (SHOPPAY shows 'Online')</t>
+          <t>Deposit and applied customer-account credit show as labeled payment rows</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -2706,24 +2558,20 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 observed for three distinct configured methods: code CASH prints 'Cash', code CHEQUE prints 'Check', code EFT prints 'EFT' - in each case the shop-configured NAME from GET /api/organizations/finance/payment-methods, not the code.</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>Clause 2 (unconfigured code, underscores to spaces) and clause 3 (SHOPPAY shows 'Online') were not produced this pass - SHOPPAY is a customer-portal payment code and cannot be recorded from the shop app. Passed on the clause that could be produced; the two unproduced clauses are listed in the not_observed field rather than assumed.</t>
-        </is>
-      </c>
+          <t>Clause 1 - INV-S2-32217 prints '(Deposit) Sep 1, 2026 - Cash   $406.09', the date being the deposit collection date, not the invoice date. Clause 2 - INV-S2-32136 prints '(Credit) Sep 7, 2026 - CM-4347   $50.00' with the full CM- prefixed number and the date the credit was applied.</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>C44948</t>
+          <t>C44949</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44948</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44949</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2733,7 +2581,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Deposit and applied customer-account credit show as labeled payment rows</t>
+          <t>Excess payment sub-line reads exactly per the credited/ to-be-credited rule</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -2743,20 +2591,24 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - INV-S2-32217 prints '(Deposit) Sep 1, 2026 - Cash   $406.09', the date being the deposit collection date, not the invoice date. Clause 2 - INV-S2-32136 prints '(Credit) Sep 7, 2026 - CM-4347   $50.00' with the full CM- prefixed number and the date the credit was applied.</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr"/>
+          <t>Produced with one EFT payment of $397.96 split across two invoices ($50.00 to INV-S2-32136, $347.96 to INV-S-31595). The sub-line printed beneath the payment row reads exactly 'of $397.96 - $347.96 will be credited' with a literal em dash. Clause 1 confirmed: it fired on a REGULAR payment spread across two invoices, not a deposit, and gated on applied &lt; full. Clause 4 confirmed: $397.96 - $50.00 = $347.96.</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Clause 2 - the 'of {full} - {excess} -&gt; Credit CM-xxxx' variant (excess already turned into a numbered credit) was not produced. Observation, not a defect: the wording 'will be credited' printed even though the excess went to a second invoice rather than to a credit. That is exactly what S8 clause 3 prescribes ('otherwise it reads...'), so the build conforms; flagging the wording as a product question, not a bug.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>C44949</t>
+          <t>C44950</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44949</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44950</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -2766,7 +2618,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Excess payment sub-line reads exactly per the credited/ to-be-credited rule</t>
+          <t>Balance equals Total minus all applied amounts, floored at $0.00</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -2776,24 +2628,24 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Produced with one EFT payment of $397.96 split across two invoices ($50.00 to INV-S2-32136, $347.96 to INV-S-31595). The sub-line printed beneath the payment row reads exactly 'of $397.96 - $347.96 will be credited' with a literal em dash. Clause 1 confirmed: it fired on a REGULAR payment spread across two invoices, not a deposit, and gated on applied &lt; full. Clause 4 confirmed: $397.96 - $50.00 = $347.96.</t>
+          <t>Clause 1 - the row is labelled exactly 'BALANCE'. Clause 2 - verified at four different states on INV-S2-32136: $746.66 (nothing applied), $546.66 (after $200.00 cash), $50.00 (after $446.66 cash + $50.00 credit CM-4347), $0.00 (after the split EFT). Every figure equals Total minus the sum of applied payments, deposits and credits.</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 - the 'of {full} - {excess} -&gt; Credit CM-xxxx' variant (excess already turned into a numbered credit) was not produced. Observation, not a defect: the wording 'will be credited' printed even though the excess went to a second invoice rather than to a credit. That is exactly what S8 clause 3 prescribes ('otherwise it reads...'), so the build conforms; flagging the wording as a product question, not a bug.</t>
+          <t>Clause 3 - the overpaid case (floored at $0.00, never negative) was not produced: the API caps an applied amount at the outstanding balance, so an over-application could not be recorded.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>C44950</t>
+          <t>C44951</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44950</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44951</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2803,7 +2655,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Balance equals Total minus all applied amounts, floored at $0.00</t>
+          <t>Paid banner appears only on portal-generated Invoice PDFs, before all content</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2813,12 +2665,12 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the row is labelled exactly 'BALANCE'. Clause 2 - verified at four different states on INV-S2-32136: $746.66 (nothing applied), $546.66 (after $200.00 cash), $50.00 (after $446.66 cash + $50.00 credit CM-4347), $0.00 (after the split EFT). Every figure equals Total minus the sum of applied payments, deposits and credits.</t>
+          <t>All five clauses observed live on staging in the customer portal (reached from the shop app account menu -&gt; Customer Portal -&gt; https://staging.portal.shopview.com), portal print menu -&gt; 'Print with Payment Receipt' (which loads /invoices/{id}/preview?include_receipt=1). (1) The banner renders before all other invoice content, above the masthead, on S-32263, S-32220, S-32052 and S-12725. (2) On S-32052 the invoice carries one shop-recorded CASH payment of $5.00 and one portal payment of $5.00: the banner lists ONLY the portal payment, and the Summary Payments section lists both ('Sep 7, 2026 - Cash $5.00' and 'Sep 7, 2026 - Online $5.00'). (3) The shop-app document for S-32263 and S-32220 - both of which now carry portal payments - contains none of the banner strings (PAID IN FULL / PARTIALLY PAID / Payment Receipt / Payments by ShopView / portal-paid-invoice-summary all zero occurrences). (4) Pill read 'PARTIALLY PAID' on S-32263 after one $100 payment and 'PAID IN FULL' after the second; 'PAID IN FULL' on S-32220, S-32264, S-12725. (5) Title read 'Payment Receipt (Batch) - Payments by ShopView' on S-32264 and S-12725 (every listed payment a batch payment) and 'Payment Receipt - Payments by ShopView' on S-32220 (one single + one batch) and on S-32263 (both single).</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>Clause 3 - the overpaid case (floored at $0.00, never negative) was not produced: the API caps an applied amount at the outstanding balance, so an over-application could not be recorded.</t>
+          <t>Portal reached via the shop app account menu -&gt; Customer Portal (POST /sso-login). Payments made with Stripe test card 4242 4242 4242 4242 in the portal's sandbox mode (is_test_mode true).</t>
         </is>
       </c>
     </row>
@@ -3175,22 +3027,22 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>C44964</t>
+          <t>C44963</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44964</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44963</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice</t>
+          <t>Estimate and Invoice Specifics</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice masthead shows 'Credit: {number}' and 'Issue date', no money</t>
+          <t>Invoice with no due date shows no Due date line; paid swap still applies</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -3200,20 +3052,24 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Read on eight credit documents produced this pass (CM-4348, CM-4350, CM-4351, CM-4352, CM-4353, CM-4354, CM-4324 and the invoice-origin CM-4355). Every one shows 'Credit: CM-nnnn' in the masthead with the CM- prefix, and 'Issue date: Sep 7, 2026' (CM-4324 correctly carries its own earlier date, Sep 2, 2026). No money figure appears in the masthead and no boxed headline figure appears anywhere on the document.</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr"/>
+          <t>Verified on work order S-17466 (customer East Moline Diesel Repair, terms Net 30) through the Estimate/Invoice toggle on the Finance tab. Toggle OFF, the Estimate: the masthead reads 'Estimate: EST-S2-17466' and 'Estimate date: Sep 6, 2026' with NO 'Due date' line anywhere - the old quirk of rendering a null due date as today's date is retired, which is clause 1. Toggle ON, the Invoice: 'Invoice: INV-S2-17466', 'Invoice date: Sep 6, 2026' and 'Due date: Oct 6, 2026', the Net 30 date correctly derived. Clause 2, the paid swap, is proven on two other records: INV-S2-32136 replaced 'Due date' with 'Paid date: Sep 6, 2026' once fully paid, and the deposit-paid INV-S2-32217 shows 'Paid date: Sep 1, 2026'.</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>CORRECTED VERDICT - the earlier Blocked was my misreading. I took 'an Invoice with no due date set' to mean a record whose due-date field is null and went looking for a data state that does not exist. The case's own phrase, 'the old quirk of rendering a null due date as today's date is retired', is taken verbatim from spec rule S10-R2, which attaches it to the ESTIMATE. The document with no due date is the Estimate view, reached with the toggle. QA lead's correction, 2026-09-07.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>C44965</t>
+          <t>C44964</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44965</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44964</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3223,7 +3079,7 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Customer address block is labeled 'Credit To' on the Credit Invoice</t>
+          <t>Credit Invoice masthead shows 'Credit: {number}' and 'Issue date', no money</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -3233,7 +3089,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the customer block is labelled 'CREDIT TO', never 'Bill To', on all eight credit documents. Clause 2 - the customer name, street, city/province and postcode all print exactly as on the Invoice. Clause 3 - no Remit Payment To block appears, and the Credit To box measures x0=60.0 to x1=535.3, i.e. 475.3pt, the full content width - the same measurement as the Invoice's Bill To.</t>
+          <t>Read on eight credit documents produced this pass (CM-4348, CM-4350, CM-4351, CM-4352, CM-4353, CM-4354, CM-4324 and the invoice-origin CM-4355). Every one shows 'Credit: CM-nnnn' in the masthead with the CM- prefix, and 'Issue date: Sep 7, 2026' (CM-4324 correctly carries its own earlier date, Sep 2, 2026). No money figure appears in the masthead and no boxed headline figure appears anywhere on the document.</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr"/>
@@ -3241,12 +3097,12 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>C44966</t>
+          <t>C44965</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44966</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44965</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3256,7 +3112,7 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Status table shows Credit Number, Status, Invoice Number correctly</t>
+          <t>Customer address block is labeled 'Credit To' on the Credit Invoice</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -3266,24 +3122,20 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the status table's columns read exactly 'CREDIT NUMBER', 'STATUS' and, when an origin invoice exists, 'INVOICE NUMBER'. Clause 2 - four of the five states were produced and each renders its own label: 'Unapplied' (CM-4348), 'Applied' (CM-4350), 'Voided' (CM-4351) and 'Partially applied' (CM-4352, CM-4324, CM-4354). Clause 3 - the invoice-origin credit CM-4355 prints 'INVOICE NUMBER  INV-S-32220'. Clause 4 - on every account-level credit (no origin invoice) the whole Invoice Number column is absent, not blank.</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t>The fifth status label, 'Refunded', was not produced: a credit refunded in part reports 'Partially applied', and a fully refunded one reports 'Applied'. Worth a look separately: the Invoice Number column prints 'INV-S-32220' while the invoice document itself is headed 'INV-S2-32220'. The case's own example uses the INV-S- form, so it is scored a pass, but the two numbers for one invoice are recorded in FINDINGS.</t>
-        </is>
-      </c>
+          <t>Clause 1 - the customer block is labelled 'CREDIT TO', never 'Bill To', on all eight credit documents. Clause 2 - the customer name, street, city/province and postcode all print exactly as on the Invoice. Clause 3 - no Remit Payment To block appears, and the Credit To box measures x0=60.0 to x1=535.3, i.e. 475.3pt, the full content width - the same measurement as the Invoice's Bill To.</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>C44967</t>
+          <t>C44966</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44967</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44966</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3293,7 +3145,7 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Credited items table shows returned parts and money-only lines correctly</t>
+          <t>Status table shows Credit Number, Status, Invoice Number correctly</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -3303,24 +3155,24 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the table's columns read exactly 'DESCRIPTION', 'QUANTITY', 'RATE', 'RESTOCKING FEE', 'TOTAL'. Clause 3 - a money-only credit line prints '--' for Quantity and '--' for Rate. Clause 4 - the Restocking Fee column is present on every credit document and reads '$0.00' where there is no fee. Clause 5 - totals are negative with a leading minus ('-$200.00', '-$40.00'), never the parentheses convention. Clause 6 - the money-only line's Description is the credit's reason where one was entered ('ZZAUTOTEST credit A'), and falls back to the memo where it was not (CM-4324 renders '100 — Admin ShopView').</t>
+          <t>Clause 1 - the status table's columns read exactly 'CREDIT NUMBER', 'STATUS' and, when an origin invoice exists, 'INVOICE NUMBER'. Clause 2 - four of the five states were produced and each renders its own label: 'Unapplied' (CM-4348), 'Applied' (CM-4350), 'Voided' (CM-4351) and 'Partially applied' (CM-4352, CM-4324, CM-4354). Clause 3 - the invoice-origin credit CM-4355 prints 'INVOICE NUMBER  INV-S-32220'. Clause 4 - on every account-level credit (no origin invoice) the whole Invoice Number column is absent, not blank.</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 - a returned part showing a negative quantity and its rate was not produced. The parts-return picker is part-sale only; a service work order's credit is a plain amount, so a part-sale invoice with lines is needed.</t>
+          <t>The fifth status label, 'Refunded', was not produced: a credit refunded in part reports 'Partially applied', and a fully refunded one reports 'Applied'. Worth a look separately: the Invoice Number column prints 'INV-S-32220' while the invoice document itself is headed 'INV-S2-32220'. The case's own example uses the INV-S- form, so it is scored a pass, but the two numbers for one invoice are recorded in FINDINGS.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>C44968</t>
+          <t>C44967</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44968</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44967</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3330,7 +3182,7 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Restocking fee reduces a returned-part credit total as specified</t>
+          <t>Credited items table shows returned parts and money-only lines correctly</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
@@ -3340,24 +3192,24 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 - on every money-only credit the Total equals the credited amount exactly (CM-4348 -$200.00, CM-4355 -$40.00, CM-4324 -$100.00).</t>
+          <t>Clause 1 - the table's columns read exactly 'DESCRIPTION', 'QUANTITY', 'RATE', 'RESTOCKING FEE', 'TOTAL'. Clause 3 - a money-only credit line prints '--' for Quantity and '--' for Rate. Clause 4 - the Restocking Fee column is present on every credit document and reads '$0.00' where there is no fee. Clause 5 - totals are negative with a leading minus ('-$200.00', '-$40.00'), never the parentheses convention. Clause 6 - the money-only line's Description is the credit's reason where one was entered ('ZZAUTOTEST credit A'), and falls back to the memo where it was not (CM-4324 renders '100 — Admin ShopView').</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the restocking-fee arithmetic (quantity -2 at $50.00 with a $10.00 fee giving -$90.00) needs a returned part, which is part-sale only and was not produced.</t>
+          <t>Clause 2 - a returned part showing a negative quantity and its rate was not produced. The parts-return picker is part-sale only; a service work order's credit is a plain amount, so a part-sale invoice with lines is needed.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>C44969</t>
+          <t>C44968</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44969</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44968</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3367,7 +3219,7 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Totals block rows and Balance follow the credit's status</t>
+          <t>Restocking fee reduces a returned-part credit total as specified</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -3377,34 +3229,34 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the totals block prints exactly 'Subtotal', 'Tax', 'Total Credit', 'Payments', 'Balance', in that order; Subtotal is the sum of the item totals and negative, Tax is a single row reading '$0.00' where no tax applies, Total Credit is negative. Clause 2 Unapplied (CM-4348) - 'Payments' shows with no rows and Balance reads $200.00 positive. Clause 3 Partially applied to an invoice (CM-4324) - 'Payments' shows with no rows and Balance reads $49.77, the open balance after $50.23 was applied. Clause 4 Applied (CM-4350) - Balance reads $0.00.</t>
+          <t>Clause 2 - on every money-only credit the Total equals the credited amount exactly (CM-4348 -$200.00, CM-4355 -$40.00, CM-4324 -$100.00).</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>Case text lags the spec on one point, and the BUILD is right: where a credit carries a refund, the Payments section DOES list rows (CM-4352 prints 'Sep 7, 2026 - Cash  -$50.00'). That is what S11-R6/R6b require since the 2026-09-04 amendment; the case still says 'the label with no rows' for partially applied. Not scored against the build.</t>
+          <t>Clause 1 - the restocking-fee arithmetic (quantity -2 at $50.00 with a $10.00 fee giving -$90.00) needs a returned part, which is part-sale only and was not produced.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>C44971</t>
+          <t>C44969</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44971</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44969</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Document Visual Standard</t>
+          <t>Credit Invoice</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Document layout matches the Design Document structure</t>
+          <t>Totals block rows and Balance follow the credit's status</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
@@ -3414,20 +3266,24 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Measured on INV-S2-32136 (2pp). Masthead: shop letterhead left (x=22-160), shop logo image centred (x=228.8-342.8, y=70-95), document block right, all sitting over a 2px ink rule (.mh border-bottom: 2px solid #121926, measured 1.5pt on paper). Bordered Addresses row (.addr-row, 1px #E3E8EF, radius 8px). Asset band with top and bottom hairlines. Order-reference chips (.ochip, bordered pills). Numbered work lines 01/02/03. 'SUMMARY' break bar (two 1.5pt ink rules either side of the label at y=556.9). Two-column tail: disclaimer left at x=60, totals right at x=280. Boxed headline figure. Three-line signature row (CUSTOMER SIGNATURE / PRINTED NAME / DATE). Single-line footer.</t>
-        </is>
-      </c>
-      <c r="G63" s="4" t="inlineStr"/>
+          <t>Clause 1 - the totals block prints exactly 'Subtotal', 'Tax', 'Total Credit', 'Payments', 'Balance', in that order; Subtotal is the sum of the item totals and negative, Tax is a single row reading '$0.00' where no tax applies, Total Credit is negative. Clause 2 Unapplied (CM-4348) - 'Payments' shows with no rows and Balance reads $200.00 positive. Clause 3 Partially applied to an invoice (CM-4324) - 'Payments' shows with no rows and Balance reads $49.77, the open balance after $50.23 was applied. Clause 4 Applied (CM-4350) - Balance reads $0.00.</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>Case text lags the spec on one point, and the BUILD is right: where a credit carries a refund, the Payments section DOES list rows (CM-4352 prints 'Sep 7, 2026 - Cash  -$50.00'). That is what S11-R6/R6b require since the 2026-09-04 amendment; the case still says 'the label with no rows' for partially applied. Not scored against the build.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>C44972</t>
+          <t>C44971</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44972</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44971</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -3437,7 +3293,7 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Only the closed palette colours appear on any document</t>
+          <t>Document layout matches the Design Document structure</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
@@ -3447,24 +3303,20 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Every vector ink on the document was extracted: text renders in #121926, #364152, #4B5565 and #257CFF only; rules render in #121926 and #CDD5DF only. #4B5565 and #CDD5DF are not palette additions - they are the print-ink floors S12-R5 names, which clamp #697586/#9AA4B2 to #4B5565 and #E3E8EF/#EEF2F6 to #CDD5DF in PDF output. The template's own S12-R2 comment lists the same closed set. No colour outside the palette-plus-floor set appears.</t>
-        </is>
-      </c>
-      <c r="G64" s="4" t="inlineStr">
-        <is>
-          <t>The only non-palette pixels in a raster of the page belong to the shop's own uploaded logo image (a greyscale bitmap in the masthead) and to text anti-aliasing. Neither is a document ink.</t>
-        </is>
-      </c>
+          <t>Measured on INV-S2-32136 (2pp). Masthead: shop letterhead left (x=22-160), shop logo image centred (x=228.8-342.8, y=70-95), document block right, all sitting over a 2px ink rule (.mh border-bottom: 2px solid #121926, measured 1.5pt on paper). Bordered Addresses row (.addr-row, 1px #E3E8EF, radius 8px). Asset band with top and bottom hairlines. Order-reference chips (.ochip, bordered pills). Numbered work lines 01/02/03. 'SUMMARY' break bar (two 1.5pt ink rules either side of the label at y=556.9). Two-column tail: disclaimer left at x=60, totals right at x=280. Boxed headline figure. Three-line signature row (CUSTOMER SIGNATURE / PRINTED NAME / DATE). Single-line footer.</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>C44973</t>
+          <t>C44972</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44973</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44972</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -3474,7 +3326,7 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Accent colour appears only on line numbers and the footer 'ShopView'</t>
+          <t>Only the closed palette colours appear on any document</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
@@ -3484,24 +3336,24 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Exactly four spans on the whole document carry the accent #257CFF: the three work-line numbers '01', '02' (page 1) and '03' (page 2), and the word 'ShopView' in the page-2 footer. Nothing else uses it - 14 accent-coloured characters in total across both pages.</t>
+          <t>Every vector ink on the document was extracted: text renders in #121926, #364152, #4B5565 and #257CFF only; rules render in #121926 and #CDD5DF only. #4B5565 and #CDD5DF are not palette additions - they are the print-ink floors S12-R5 names, which clamp #697586/#9AA4B2 to #4B5565 and #E3E8EF/#EEF2F6 to #CDD5DF in PDF output. The template's own S12-R2 comment lists the same closed set. No colour outside the palette-plus-floor set appears.</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 (Parts Sale, accent on 'ShopView' only) belongs to the Parts Sale document and is recorded under that section.</t>
+          <t>The only non-palette pixels in a raster of the page belong to the shop's own uploaded logo image (a greyscale bitmap in the masthead) and to text anti-aliasing. Neither is a document ink.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>C44975</t>
+          <t>C44973</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44975</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44973</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -3511,7 +3363,7 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Print/PDF ink floor keeps text and rules dark enough</t>
+          <t>Accent colour appears only on line numbers and the footer 'ShopView'</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -3521,20 +3373,24 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the lightest text ink anywhere on the document is #4B5565; nothing lighter appears. Clause 2 - the only text below 10px is at 9.5px and 9.0px and both render #364152, not lighter. Clause 3 - every hairline rule renders #CDD5DF (0.75pt stroke), the floor value exactly.</t>
-        </is>
-      </c>
-      <c r="G66" s="4" t="inlineStr"/>
+          <t>Exactly four spans on the whole document carry the accent #257CFF: the three work-line numbers '01', '02' (page 1) and '03' (page 2), and the word 'ShopView' in the page-2 footer. Nothing else uses it - 14 accent-coloured characters in total across both pages.</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>Clause 2 (Parts Sale, accent on 'ShopView' only) belongs to the Parts Sale document and is recorded under that section.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>C44976</t>
+          <t>C44975</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44976</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44975</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3544,7 +3400,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Every document is fully legible in grayscale</t>
+          <t>Print/PDF ink floor keeps text and rules dark enough</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
@@ -3554,7 +3410,7 @@
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 both halves observed. Credit amounts carry the leading minus: the Credit document CM-4347 prints 'Subtotal -$50.00' and 'Total Credit -$50.00'. Discounts carry parentheses: INV-S2-32219 prints the work-order-wide discount as 'ZZAUTOTEST Loyalty Discount  ($15.00)'. Clause 1 - grayscale legibility follows from C44975: the document uses no colour to carry meaning, the lightest ink is #4B5565 and the lightest rule #CDD5DF, so nothing depends on hue.</t>
+          <t>Clause 1 - the lightest text ink anywhere on the document is #4B5565; nothing lighter appears. Clause 2 - the only text below 10px is at 9.5px and 9.0px and both render #364152, not lighter. Clause 3 - every hairline rule renders #CDD5DF (0.75pt stroke), the floor value exactly.</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr"/>
@@ -3562,12 +3418,12 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>C44977</t>
+          <t>C44976</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44977</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44976</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -3577,7 +3433,7 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Prototype chrome does not appear on any real document</t>
+          <t>Every document is fully legible in grayscale</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -3587,7 +3443,7 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>The template carries no box-shadow declaration at all, and no toggle, settings or theme control markup - the design prototype's control strips are absent from the rendered document. The PDF is a plain white sheet with no drop shadow and no rounded sheet corners; the only border-radius values in the document CSS are 8px on the Addresses box and 6px on the order-reference chips, both of which are design elements rather than sheet presentation.</t>
+          <t>Clause 2 both halves observed. Credit amounts carry the leading minus: the Credit document CM-4347 prints 'Subtotal -$50.00' and 'Total Credit -$50.00'. Discounts carry parentheses: INV-S2-32219 prints the work-order-wide discount as 'ZZAUTOTEST Loyalty Discount  ($15.00)'. Clause 1 - grayscale legibility follows from C44975: the document uses no colour to carry meaning, the lightest ink is #4B5565 and the lightest rule #CDD5DF, so nothing depends on hue.</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr"/>
@@ -3595,12 +3451,12 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>C44978</t>
+          <t>C44977</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44978</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44977</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -3610,7 +3466,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Work-section rules and dividers follow the specified treatment</t>
+          <t>Prototype chrome does not appear on any real document</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
@@ -3620,7 +3476,7 @@
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the work section opens with a 2px ink rule (.job-first border-top-width: 2px over .job border-top: 1px solid #121926; measured 1.5pt #121926 on paper). Clause 2 - numbered jobs are separated by a 1px ink #121926 rule. Clause 3 - charge rows inside a job are ruled with #EEF2F6 dividers (.work-summary-table-new tr.crow td), printed at the #CDD5DF floor. Clause 4 - the 'Labor' and 'Parts' sub-section labels carry no border declaration and none renders. Clause 5 measured on INV-S2-32219: charge row at y=459.7, adjustment row at y=480.2, divider at y=494.3 - the divider follows the last adjustment row and never sits between the line and its adjustments.</t>
+          <t>The template carries no box-shadow declaration at all, and no toggle, settings or theme control markup - the design prototype's control strips are absent from the rendered document. The PDF is a plain white sheet with no drop shadow and no rounded sheet corners; the only border-radius values in the document CSS are 8px on the Addresses box and 6px on the order-reference chips, both of which are design elements rather than sheet presentation.</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr"/>
@@ -3628,12 +3484,12 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>C44979</t>
+          <t>C44978</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44979</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44978</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -3643,7 +3499,7 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Section labels use the three-tier hierarchy with exact sizes and inks</t>
+          <t>Work-section rules and dividers follow the specified treatment</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
@@ -3653,34 +3509,30 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Measured on INV-S2-32136. Clause 1 - 'WORK PERFORMED' renders at 11.0px bold. Clause 2 - 'SCOPE OF WORK' at 10.0px bold. Clause 3 - the in-job 'LABOR' and 'PARTS' labels at 10.5px bold. Clause 4 - all three sit below the job titles, which render at 16.0px bold. Inks follow the print floor (C44975).</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>Weight cannot be discriminated beyond regular-vs-bold in the PDF because only two faces are embedded - that is the C44974 failure, not a separate one here. Sizes, which are what this case pins, are all exact.</t>
-        </is>
-      </c>
+          <t>Clause 1 - the work section opens with a 2px ink rule (.job-first border-top-width: 2px over .job border-top: 1px solid #121926; measured 1.5pt #121926 on paper). Clause 2 - numbered jobs are separated by a 1px ink #121926 rule. Clause 3 - charge rows inside a job are ruled with #EEF2F6 dividers (.work-summary-table-new tr.crow td), printed at the #CDD5DF floor. Clause 4 - the 'Labor' and 'Parts' sub-section labels carry no border declaration and none renders. Clause 5 measured on INV-S2-32219: charge row at y=459.7, adjustment row at y=480.2, divider at y=494.3 - the divider follows the last adjustment row and never sits between the line and its adjustments.</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>C44980</t>
+          <t>C44979</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44980</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44979</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Parts Sale Estimate and Invoice</t>
+          <t>Document Visual Standard</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Parts Sale documents behave as the Estimate/Invoice except as stated</t>
+          <t>Section labels use the three-tier hierarchy with exact sizes and inks</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -3690,20 +3542,24 @@
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Both documents rendered for part sale P2-1931 and for P2-1930. The Parts Sale Estimate behaves as the Estimate: 'Estimate: EST-P2-1931', 'Estimate date: Sep 7, 2026', boxed 'ESTIMATED TOTAL $186.90', no Payments block and no Balance. The Parts Sale Invoice behaves as the Invoice: 'Invoice: INV-P2-1931', 'Invoice date' and 'Due date: Sep 14, 2026', 'Payments' and 'BALANCE $186.90'. Masthead, Addresses (Bill To at full width, no Remit Payment To), financial summary, disclaimer, three-line signature row, footer and the whole visual standard match the Invoice. The Story 13 departures are the only differences and are recorded case by case below.</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="inlineStr"/>
+          <t>Measured on INV-S2-32136. Clause 1 - 'WORK PERFORMED' renders at 11.0px bold. Clause 2 - 'SCOPE OF WORK' at 10.0px bold. Clause 3 - the in-job 'LABOR' and 'PARTS' labels at 10.5px bold. Clause 4 - all three sit below the job titles, which render at 16.0px bold. Inks follow the print floor (C44975).</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>Weight cannot be discriminated beyond regular-vs-bold in the PDF because only two faces are embedded - that is the C44974 failure, not a separate one here. Sizes, which are what this case pins, are all exact.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>C44981</t>
+          <t>C44980</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44981</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44980</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3713,7 +3569,7 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Parts Sale body is a single flat 'Parts' section, no jobs</t>
+          <t>Parts Sale documents behave as the Estimate/Invoice except as stated</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -3723,24 +3579,20 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>CORRECTED VERDICT - the earlier Failed was wrong. Re-tested on part sale P2-1931 after reading its own per-view settings: the 'Part number' toggle was OFF on that document, which is why the number was absent. With all four Parts Sale toggles ON the line renders 'P550848 - FUEL/WATER SEPARATOR, (FS19732, 33732, BF1385-SPS)  2  $80.00  $160.00' - part number, description, quantity, rate and amount, exactly as S13-R2 requires. Clause 1: the body is a single section headed 'PARTS'. Clause 3: no job blocks, no line numbers, no 'Scope of work', no Labor section and no Declined Work section.</t>
-        </is>
-      </c>
-      <c r="G72" s="4" t="inlineStr">
-        <is>
-          <t>The Parts Sale settings panel carries four toggles, not the Invoice's nine - Part number, Part quantity, Part price, Part description - which is consistent with a parts-only document having no labor fields. Ticket SV-9774 was raised on the earlier wrong reading and has been obsoleted by the QA lead.</t>
-        </is>
-      </c>
+          <t>Both documents rendered for part sale P2-1931 and for P2-1930. The Parts Sale Estimate behaves as the Estimate: 'Estimate: EST-P2-1931', 'Estimate date: Sep 7, 2026', boxed 'ESTIMATED TOTAL $186.90', no Payments block and no Balance. The Parts Sale Invoice behaves as the Invoice: 'Invoice: INV-P2-1931', 'Invoice date' and 'Due date: Sep 14, 2026', 'Payments' and 'BALANCE $186.90'. Masthead, Addresses (Bill To at full width, no Remit Payment To), financial summary, disclaimer, three-line signature row, footer and the whole visual standard match the Invoice. The Story 13 departures are the only differences and are recorded case by case below.</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>C44982</t>
+          <t>C44981</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44982</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44981</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -3750,7 +3602,7 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Parts Sale line-level fees/discounts render as on the Invoice</t>
+          <t>Parts Sale body is a single flat 'Parts' section, no jobs</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -3760,20 +3612,24 @@
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>A line-level fee of $9.00 x qty 2 = $18.00 was added to the part on P2-1931. Clause 1 - it renders indented under its part line as '↳ ZZAUTOTEST Part Handling Fee   $18.00', exactly as on the Invoice. Clause 2 - measured: the part row band ends at y=361.9 and the divider (0.75pt #CDD5DF) sits at y=361.9, below the adjustment row, never between the part and its adjustment.</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr"/>
+          <t>CORRECTED VERDICT - the earlier Failed was wrong. Re-tested on part sale P2-1931 after reading its own per-view settings: the 'Part number' toggle was OFF on that document, which is why the number was absent. With all four Parts Sale toggles ON the line renders 'P550848 - FUEL/WATER SEPARATOR, (FS19732, 33732, BF1385-SPS)  2  $80.00  $160.00' - part number, description, quantity, rate and amount, exactly as S13-R2 requires. Clause 1: the body is a single section headed 'PARTS'. Clause 3: no job blocks, no line numbers, no 'Scope of work', no Labor section and no Declined Work section.</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>The Parts Sale settings panel carries four toggles, not the Invoice's nine - Part number, Part quantity, Part price, Part description - which is consistent with a parts-only document having no labor fields. Ticket SV-9774 was raised on the earlier wrong reading and has been obsoleted by the QA lead.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>C44983</t>
+          <t>C44982</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44983</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44982</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -3783,7 +3639,7 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Parts Sale document number keeps parts-sale numbering</t>
+          <t>Parts Sale line-level fees/discounts render as on the Invoice</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
@@ -3793,7 +3649,7 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Parts-sale numbering is carried through on both records and both document types: 'Estimate: EST-P2-1931' / 'Invoice: INV-P2-1931', and 'Estimate: EST-P2-1930' / 'Invoice: INV-P2-1930'.</t>
+          <t>A line-level fee of $9.00 x qty 2 = $18.00 was added to the part on P2-1931. Clause 1 - it renders indented under its part line as '↳ ZZAUTOTEST Part Handling Fee   $18.00', exactly as on the Invoice. Clause 2 - measured: the part row band ends at y=361.9 and the divider (0.75pt #CDD5DF) sits at y=361.9, below the adjustment row, never between the part and its adjustment.</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr"/>
@@ -3801,12 +3657,12 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>C44984</t>
+          <t>C44983</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44984</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44983</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -3816,7 +3672,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Parts Sale reference fields drop Work Order and Approval Code</t>
+          <t>Parts Sale document number keeps parts-sale numbering</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -3826,7 +3682,7 @@
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - neither the Work Order field nor the Approval Code field appears on any of the four parts sale documents rendered. Clause 2 - 'Terms' always shows ('Terms  Net 7' on P2-1931, 'Terms  COD' on P2-1930); Customer PO behaves as on the Invoice, printing when set and absent when not. Clause 3 - the Authorizer follows the parts-sale treatment, verified in full under C44985.</t>
+          <t>Parts-sale numbering is carried through on both records and both document types: 'Estimate: EST-P2-1931' / 'Invoice: INV-P2-1931', and 'Estimate: EST-P2-1930' / 'Invoice: INV-P2-1930'.</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr"/>
@@ -3834,12 +3690,12 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>C44985</t>
+          <t>C44984</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44985</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44984</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -3849,7 +3705,7 @@
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Parts sale receives the Authorizer treatment (net-new)</t>
+          <t>Parts Sale reference fields drop Work Order and Approval Code</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
@@ -3859,20 +3715,24 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>All four clauses driven live on part sale P2-1931. Clause 1 - the Authorizer is empty by default: the first render carried no Authorizer row at all. Clause 4 - once set to the customer's 'Approves Work' contact, the document prints 'Authorizer  Savannah Tran' in the reference row. Clause 2 - with the parts sale invoiced, changing the authorizer is refused: HTTP 409 'The authorizer cannot be changed on an invoiced or paid work order'. Clause 3 - after reversing that invoice the same change succeeds (HTTP 200), so the field becomes editable again, mirroring S3-R8.</t>
-        </is>
-      </c>
-      <c r="G76" s="4" t="inlineStr"/>
+          <t>Clause 1 - neither the Work Order field nor the Approval Code field appears on any of the four parts sale documents rendered. Clause 2 - 'Terms' always shows ('Terms Net 7' on P2-1931, 'Terms COD' on P2-1930); Customer PO behaves as on the Invoice, printing when set and absent when not. Clause 3 - the Authorizer follows the parts-sale treatment.</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>STRENGTHENED by the 2026-09-07 rewrite of S3-N1. Clause 1 used to rest on a Story 13 statement alone; the rewritten S3-N1 now names this case explicitly as hide-case (a): 'The document has no work order behind it. A standalone Parts Sale Estimate or Parts Sale Invoice has none, so the field is omitted there: no label and no empty value area.' The observation is unchanged and is now directly cited.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>C44986</t>
+          <t>C44985</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44986</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44985</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -3882,7 +3742,7 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Parts Sale financial summary shows no Labor and no Shop supplies row</t>
+          <t>Parts sale receives the Authorizer treatment (net-new)</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
@@ -3892,7 +3752,7 @@
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - the financial summary on both P2-1931 and P2-1930 shows no 'Labor' row and no 'Shop supplies' row. Clause 2 - the rows present are identical in label and treatment to the Invoice: 'Parts $160.00', 'Adjustments' with its 'Parts $18.00' rollup, 'Subtotal $178.00', 'GST (5%) $8.90', 'Total $186.90', 'Payments', 'BALANCE $186.90'. Arithmetic reconciles: 160.00 + 18.00 = 178.00; 5% of 178.00 = 8.90; 178.00 + 8.90 = 186.90.</t>
+          <t>All four clauses driven live on part sale P2-1931. Clause 1 - the Authorizer is empty by default: the first render carried no Authorizer row at all. Clause 4 - once set to the customer's 'Approves Work' contact, the document prints 'Authorizer  Savannah Tran' in the reference row. Clause 2 - with the parts sale invoiced, changing the authorizer is refused: HTTP 409 'The authorizer cannot be changed on an invoiced or paid work order'. Clause 3 - after reversing that invoice the same change succeeds (HTTP 200), so the field becomes editable again, mirroring S3-R8.</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
@@ -3900,12 +3760,12 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>C44987</t>
+          <t>C44986</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44987</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44986</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -3915,7 +3775,7 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Batch and imported invoices are out of scope (kept on current templates)</t>
+          <t>Parts Sale financial summary shows no Labor and no Shop supplies row</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -3925,34 +3785,30 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Rendered a batch PDF (POST /api/invoices/batch-pdf over two of this pass's invoices). It comes back entirely on the OLD template and is not half-restyled: the typeface is Nunito Sans throughout, the labels are the pre-refresh ones ('Invoice Date:' with a capital D, 'Bill To' in title case, 'Parts Order', a Description/Quantity/Rate/Amount table header), and none of the refresh markers appears - no accent-coloured line numbers, no order-reference chips, no 'WORK PERFORMED' section head, no boxed headline figure. Clauses 1, 2 and 3 all hold.</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>An imported work order's document was not rendered this pass; the batch path alone was exercised. Side evidence for SV-9761: the OLD template's Nunito Sans IS embedded correctly, while the refreshed template asks for Inter and silently falls back to DejaVu Sans. The font is missing from the refreshed pipeline, not from the image generally.</t>
-        </is>
-      </c>
+          <t>Clause 1 - the financial summary on both P2-1931 and P2-1930 shows no 'Labor' row and no 'Shop supplies' row. Clause 2 - the rows present are identical in label and treatment to the Invoice: 'Parts $160.00', 'Adjustments' with its 'Parts $18.00' rollup, 'Subtotal $178.00', 'GST (5%) $8.90', 'Total $186.90', 'Payments', 'BALANCE $186.90'. Arithmetic reconciles: 160.00 + 18.00 = 178.00; 5% of 178.00 = 8.90; 178.00 + 8.90 = 186.90.</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>C45168</t>
+          <t>C44987</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45168</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/44987</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice never shows Remit Payment To and Credit To spans full width</t>
+          <t>Batch and imported invoices are out of scope (kept on current templates)</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -3962,30 +3818,34 @@
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Both clauses. No 'Remit Payment To' block anywhere on the Credit Invoice, and the 'CREDIT TO' card measures x0=60.0 -&gt; x1=535.3 = 475.3pt, the full content width (page.get_drawings()).</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr"/>
+          <t>Rendered a batch PDF (POST /api/invoices/batch-pdf over two of this pass's invoices). It comes back entirely on the OLD template and is not half-restyled: the typeface is Nunito Sans throughout, the labels are the pre-refresh ones ('Invoice Date:' with a capital D, 'Bill To' in title case, 'Parts Order', a Description/Quantity/Rate/Amount table header), and none of the refresh markers appears - no accent-coloured line numbers, no order-reference chips, no 'WORK PERFORMED' section head, no boxed headline figure. Clauses 1, 2 and 3 all hold.</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>An imported work order's document was not rendered this pass; the batch path alone was exercised. Side evidence for SV-9761: the OLD template's Nunito Sans IS embedded correctly, while the refreshed template asks for Inter and silently falls back to DejaVu Sans. The font is missing from the refreshed pipeline, not from the image generally.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>C45169</t>
+          <t>C45168</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45169</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45168</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>API — Authorizer Entry</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Authorizer change is rejected by the API while a non-voided invoice exists</t>
+          <t>Credit Invoice never shows Remit Payment To and Credit To spans full width</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -3995,7 +3855,7 @@
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - POST /api/work-orders/change-authorizer against invoiced work order S2-32221 returns HTTP 409, 'The authorizer cannot be changed on an invoiced or paid work order', and a live re-read shows authorizer_full_name still null: the server-side lock cannot be bypassed. The same 409 was reproduced independently on the invoiced parts sale P2-1931. Clause 2 - the lock is conditional, not permanent: after reversing that parts sale's invoice the identical call returned HTTP 200 and the change landed.</t>
+          <t>Both clauses. No 'Remit Payment To' block anywhere on the Credit Invoice, and the 'CREDIT TO' card measures x0=60.0 -&gt; x1=535.3 = 475.3pt, the full content width (page.get_drawings()).</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr"/>
@@ -4003,12 +3863,12 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>C45170</t>
+          <t>C45169</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45170</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45169</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -4018,7 +3878,7 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Authorizer API rejects a non-approver or another company's contact</t>
+          <t>Authorizer change is rejected by the API while a non-voided invoice exists</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
@@ -4028,34 +3888,30 @@
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Both rejections driven live against un-invoiced work order S2-32222. (a) A contact of the SAME customer created without 'Approves Work' (ZZAUTOTEST NonApprover) is refused: HTTP 422, 'The contact ... cannot be used as the authorizer for this work order.' (b) ANOTHER company's contact, one that does carry 'Approves Work' (7 Star Truck Repair), is refused with the same 422. After both attempts a live re-read shows authorizer_full_name still null - unchanged in each case. Only a contact of this customer with 'Approves Work' enabled is accepted, which the positive path proved separately.</t>
-        </is>
-      </c>
-      <c r="G81" s="4" t="inlineStr">
-        <is>
-          <t>The cross-company contact answers 422 rather than 404; the case allows either.</t>
-        </is>
-      </c>
+          <t>Clause 1 - POST /api/work-orders/change-authorizer against invoiced work order S2-32221 returns HTTP 409, 'The authorizer cannot be changed on an invoiced or paid work order', and a live re-read shows authorizer_full_name still null: the server-side lock cannot be bypassed. The same 409 was reproduced independently on the invoiced parts sale P2-1931. Clause 2 - the lock is conditional, not permanent: after reversing that parts sale's invoice the identical call returned HTTP 200 and the change landed.</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>C45171</t>
+          <t>C45170</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45171</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45170</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Asset Section</t>
+          <t>API — Authorizer Entry</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Asset section is hidden when the work order has no asset attached</t>
+          <t>Authorizer API rejects a non-approver or another company's contact</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -4065,30 +3921,34 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Part sale P2-1931 has no asset attached - the live record reads vehicle.id = null - and its invoice INV-P2-1931 has no asset band at all. The document runs straight from the ADDRESSES block to the order-reference chips and then to PARTS: no 'ASSET' heading, no empty labels, nothing left behind.</t>
-        </is>
-      </c>
-      <c r="G82" s="4" t="inlineStr"/>
+          <t>Both rejections driven live against un-invoiced work order S2-32222. (a) A contact of the SAME customer created without 'Approves Work' (ZZAUTOTEST NonApprover) is refused: HTTP 422, 'The contact ... cannot be used as the authorizer for this work order.' (b) ANOTHER company's contact, one that does carry 'Approves Work' (7 Star Truck Repair), is refused with the same 422. After both attempts a live re-read shows authorizer_full_name still null - unchanged in each case. Only a contact of this customer with 'Approves Work' enabled is accepted, which the positive path proved separately.</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>The cross-company contact answers 422 rather than 404; the case allows either.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>C45172</t>
+          <t>C45171</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45172</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45171</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Work Section</t>
+          <t>Asset Section</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Summarize labor total and Summarize parts total control the line footer figures</t>
+          <t>Asset section is hidden when the work order has no asset attached</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
@@ -4098,7 +3958,7 @@
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Measured on WO S2-32136 through the Finance tab's own settings panel. Clause 1, 'Summarize labor total' off: the footer 'Labor' figure disappears while 'Parts $48.31' and 'Line total $198.26' remain. Clause 2, both summarize settings off: the footer shows 'Line total $198.26' standing alone AND the vertical divider is genuinely gone - the element's class changes from 'ltot with-divider' to plain 'ltot' on all three lines, and it changes back when the settings are restored. Clause 3: 'Line total' is present in every one of the four states tested.</t>
+          <t>Part sale P2-1931 has no asset attached - the live record reads vehicle.id = null - and its invoice INV-P2-1931 has no asset band at all. The document runs straight from the ADDRESSES block to the order-reference chips and then to PARTS: no 'ASSET' heading, no empty labels, nothing left behind.</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr"/>
@@ -4106,12 +3966,12 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>C45173</t>
+          <t>C45172</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45173</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45172</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4121,7 +3981,7 @@
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Line numbers move to three digits from line 100 on a large document</t>
+          <t>Summarize labor total and Summarize parts total control the line footer figures</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -4131,34 +3991,30 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Seeded work order S2-32231 with 105 authorised lines and rendered it. Clause 1: line numbers 01 to 99 print as two digits and 100 to 105 print as three - all 105 numbers were extracted from the document and checked in sequence, with the two-to-three digit change happening exactly at 100. Clause 2: the render returned HTTP 200 in 3.5 seconds and produced a well-formed 19-page PDF - no timeout, no truncation.</t>
-        </is>
-      </c>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>Observation for the QA lead, not a finding: at 105 lines the labour total reaches $36,750.00 and the summary prints 'Shop supplies (10.5% of labor)  $350.00'. The $350.00 is correct - the location's maximum shop-supplies charge is $350 and the cap binds - and the spec sanctions the cap explicitly ('an optional maximum charge amount'), so this is spec-conformant. But the label still advertises a percentage that does not reconcile with the amount (10.5% of $36,750 is $3,858.75), which a customer could reasonably query. Worth a product decision on whether the percentage should be suppressed once the cap binds.</t>
-        </is>
-      </c>
+          <t>Measured on WO S2-32136 through the Finance tab's own settings panel. Clause 1, 'Summarize labor total' off: the footer 'Labor' figure disappears while 'Parts $48.31' and 'Line total $198.26' remain. Clause 2, both summarize settings off: the footer shows 'Line total $198.26' standing alone AND the vertical divider is genuinely gone - the element's class changes from 'ltot with-divider' to plain 'ltot' on all three lines, and it changes back when the settings are restored. Clause 3: 'Line total' is present in every one of the four states tested.</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>C45174</t>
+          <t>C45173</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45174</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45173</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Paid Banner, Payments and Balance</t>
+          <t>Work Section</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>A fully reversed payment does not appear in the Payments section</t>
+          <t>Line numbers move to three digits from line 100 on a large document</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -4168,30 +4024,34 @@
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>After reversing the $546.66 cheque the Payments section lists only the surviving 'Sep 5, 2026 - Cash $200.00' row; the reversed payment is absent entirely. BALANCE $546.66 = $746.66 total minus the one applied amount.</t>
-        </is>
-      </c>
-      <c r="G85" s="4" t="inlineStr"/>
+          <t>Seeded work order S2-32231 with 105 authorised lines and rendered it. Clause 1: line numbers 01 to 99 print as two digits and 100 to 105 print as three - all 105 numbers were extracted from the document and checked in sequence, with the two-to-three digit change happening exactly at 100. Clause 2: the render returned HTTP 200 in 3.5 seconds and produced a well-formed 19-page PDF - no timeout, no truncation.</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Observation for the QA lead, not a finding: at 105 lines the labour total reaches $36,750.00 and the summary prints 'Shop supplies (10.5% of labor)  $350.00'. The $350.00 is correct - the location's maximum shop-supplies charge is $350 and the cap binds - and the spec sanctions the cap explicitly ('an optional maximum charge amount'), so this is spec-conformant. But the label still advertises a percentage that does not reconcile with the amount (10.5% of $36,750 is $3,858.75), which a customer could reasonably query. Worth a product decision on whether the percentage should be suppressed once the cap binds.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>C45176</t>
+          <t>C45174</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45176</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45174</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Estimate and Invoice Specifics</t>
+          <t>Paid Banner, Payments and Balance</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Paid date is the most recent applied row and may fall before the invoice date</t>
+          <t>A fully reversed payment does not appear in the Payments section</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
@@ -4201,7 +4061,7 @@
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - INV-S2-32217: deposit DEP-4704 of $406.09 collected 1 Sep, invoice created 7 Sep, auto-applied in full; masthead prints 'Invoice date: Sep 7, 2026' / 'Paid date: Sep 1, 2026' - the earlier date shown as-is. Clause 2 - INV-S2-32136 paid by two payments (Sep 5 Cash $200.00, Sep 6 Check $546.66): 'Paid date: Sep 6, 2026', the LATEST applied date.</t>
+          <t>After reversing the $546.66 cheque the Payments section lists only the surviving 'Sep 5, 2026 - Cash $200.00' row; the reversed payment is absent entirely. BALANCE $546.66 = $746.66 total minus the one applied amount.</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr"/>
@@ -4209,22 +4069,22 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>C45177</t>
+          <t>C45175</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45177</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45175</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Estimate and Invoice Specifics</t>
+          <t>Paid Banner, Payments and Balance</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Reversing a payment returns the masthead to Due date</t>
+          <t>Paid banner pill and title wording follow the paid state and the batch rule</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -4234,30 +4094,34 @@
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>INV-S2-32136 was fully paid showing 'Paid date: Sep 6, 2026'. Reversing the $546.66 cheque re-rendered the masthead as 'Invoice date: Sep 7, 2026' / 'Due date: Sep 14, 2026' with no Paid date, and BALANCE returned to $546.66 - the label is decided at render time.</t>
-        </is>
-      </c>
-      <c r="G87" s="4" t="inlineStr"/>
+          <t>All three clauses observed live in the customer portal on staging. (1) Fully paid -&gt; pill reads exactly 'PAID IN FULL' (S-32220, S-32264, S-32263 after its second payment, S-12725); partially paid -&gt; exactly 'PARTIALLY PAID' (S-32263 after one $100 payment of $406.09, S-32052 with $10.00 of $17.45 paid). (2) Title reads exactly 'Payment Receipt - Payments by ShopView' whenever any listed payment is a single payment - S-32263 (two singles) and S-32220 (one single + one batch). (3) When every listed payment is a batch payment the title reads exactly 'Payment Receipt (Batch) - Payments by ShopView' - S-32264 (batch of two invoices) and S-12725 (batch of two invoices, paid Apr 17 2026).</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>Portal reached from the shop app account menu -&gt; Customer Portal; document taken from the portal print menu -&gt; 'Print with Payment Receipt'.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>C45179</t>
+          <t>C45176</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45179</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45176</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice</t>
+          <t>Estimate and Invoice Specifics</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice Balance shows the full open balance on an unapplied credit</t>
+          <t>Paid date is the most recent applied row and may fall before the invoice date</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -4267,7 +4131,7 @@
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>CM-4348 immediately after creation, unapplied: 'Payments' shows the label with no rows beneath it, and 'Balance' reads $200.00 - positive, the credit's full open balance. Not $0.00.</t>
+          <t>Clause 1 - INV-S2-32217: deposit DEP-4704 of $406.09 collected 1 Sep, invoice created 7 Sep, auto-applied in full; masthead prints 'Invoice date: Sep 7, 2026' / 'Paid date: Sep 1, 2026' - the earlier date shown as-is. Clause 2 - INV-S2-32136 paid by two payments (Sep 5 Cash $200.00, Sep 6 Check $546.66): 'Paid date: Sep 6, 2026', the LATEST applied date.</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr"/>
@@ -4275,22 +4139,22 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>C45180</t>
+          <t>C45177</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45180</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45177</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice</t>
+          <t>Estimate and Invoice Specifics</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Credit Balance shows the remaining open balance when partly applied</t>
+          <t>Reversing a payment returns the masthead to Due date</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
@@ -4300,34 +4164,30 @@
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>CM-4324 ($100.00 credit) applied against invoice S-32220 whose remaining balance was only $50.23, so only part of the credit was consumed. The document shows 'Payments' with no rows - the application to the invoice is not listed - and 'Balance  $49.77', positive, the original $100.00 minus the $50.23 applied.</t>
-        </is>
-      </c>
-      <c r="G89" s="4" t="inlineStr">
-        <is>
-          <t>The case's illustrative figures are $200/$120; the same rule was exercised at $100.00/$49.77 because the API applies the whole available credit unless the invoice balance caps it.</t>
-        </is>
-      </c>
+          <t>INV-S2-32136 was fully paid showing 'Paid date: Sep 6, 2026'. Reversing the $546.66 cheque re-rendered the masthead as 'Invoice date: Sep 7, 2026' / 'Due date: Sep 14, 2026' with no Paid date, and BALANCE returned to $546.66 - the label is decided at render time.</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>C45181</t>
+          <t>C45178</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45181</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45178</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice</t>
+          <t>Estimate and Invoice Specifics</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Credit Balance reads $0.00 when fully applied and when voided</t>
+          <t>A zero-total invoice with nothing applied is not treated as fully paid</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -4337,7 +4197,7 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - CM-4350, fully applied against S-32219: Balance reads $0.00. Clause 2 - CM-4351, voided: Balance reads $0.00, the items table and the totals block render exactly as on the unapplied credits (Subtotal -$200.00, Tax $0.00, Total Credit -$200.00), and the word 'Voided' in the status table is the only indication of the state.</t>
+          <t>Seeded work order S2-32262 with a $350.00 line and a work-order-wide discount of $386.75, giving Subtotal $0.00, GST $0.00 and Total $0.00 with nothing applied (the invoice-create response confirms auto_paid false and no payment, deposit or credit rows). Clause 1: the masthead reads 'Invoice date: Sep 7, 2026' and 'Due date: Sep 14, 2026' - a Due date, NOT a Paid date. Clause 2 holds by construction: Balance is $0.00 but no row has been applied, and the invoice is correctly not treated as fully paid.</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr"/>
@@ -4345,12 +4205,12 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>C45182</t>
+          <t>C45179</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45182</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45179</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -4360,7 +4220,7 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice lists refund rows and the open balance until consumed</t>
+          <t>Credit Invoice Balance shows the full open balance on an unapplied credit</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -4370,24 +4230,20 @@
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - CM-4352, $50.00 cashed out: the Payments section lists 'Sep 7, 2026 - Cash   -$50.00', the '{date} - {method}' shape with a negative amount. Clause 2 - its Balance reads $150.00, positive. Clause 3 - CM-4353, fully consumed ($50.00 refunded then the remaining $150.00 applied): the Payments section lists both rows ('Sep 7, 2026 - Cash  -$50.00' and 'Sep 7, 2026 - Applied  -$150.00') and Balance reads $0.00.</t>
-        </is>
-      </c>
-      <c r="G91" s="4" t="inlineStr">
-        <is>
-          <t>No regression against the shipped SV-7754 rendering.</t>
-        </is>
-      </c>
+          <t>CM-4348 immediately after creation, unapplied: 'Payments' shows the label with no rows beneath it, and 'Balance' reads $200.00 - positive, the credit's full open balance. Not $0.00.</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>C45183</t>
+          <t>C45180</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45183</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45180</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -4397,7 +4253,7 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Credit Balance is correct when partly refunded and partly applied</t>
+          <t>Credit Balance shows the remaining open balance when partly applied</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
@@ -4407,30 +4263,34 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>CM-4354 built to the case's exact figures: a $200.00 credit, $50.00 cashed out and $80.00 applied to invoice S-31595. The document lists both consumption rows and 'Balance  $70.00', positive - the original credit total minus the amount refunded minus the amount applied.</t>
-        </is>
-      </c>
-      <c r="G92" s="4" t="inlineStr"/>
+          <t>CM-4324 ($100.00 credit) applied against invoice S-32220 whose remaining balance was only $50.23, so only part of the credit was consumed. The document shows 'Payments' with no rows - the application to the invoice is not listed - and 'Balance  $49.77', positive, the original $100.00 minus the $50.23 applied.</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>The case's illustrative figures are $200/$120; the same rule was exercised at $100.00/$49.77 because the API applies the whole available credit unless the invoice balance caps it.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>C45184</t>
+          <t>C45181</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45184</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45181</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Cross-Cutting and Regression</t>
+          <t>Credit Invoice</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Every date on every document renders in the fixed Jan 5, 2026 format</t>
+          <t>Credit Balance reads $0.00 when fully applied and when voided</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -4440,34 +4300,30 @@
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - every date across all 25 documents captured this pass renders in the 'Mon D, YYYY' style: Sep 1, Sep 2, Sep 5, Sep 6, Sep 7, Sep 14, Jul 28, Jul 30 2026. Scanned for other date shapes (d/m/y, ISO) and for leading zeros - none found anywhere. Clause 3 - the only 'Date / Time' field is the paid banner's, which is not present on any shop-app document.</t>
-        </is>
-      </c>
-      <c r="G93" s="4" t="inlineStr">
-        <is>
-          <t>Clause 2's US half: all three workplaces in this organisation are Canadian (Calgary, Lethbridge, Toronto), so a US shop could not be rendered to prove the format does not change.</t>
-        </is>
-      </c>
+          <t>Clause 1 - CM-4350, fully applied against S-32219: Balance reads $0.00. Clause 2 - CM-4351, voided: Balance reads $0.00, the items table and the totals block render exactly as on the unapplied credits (Subtotal -$200.00, Tax $0.00, Total Credit -$200.00), and the word 'Voided' in the status table is the only indication of the state.</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>C45185</t>
+          <t>C45182</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45185</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45182</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Cross-Cutting and Regression</t>
+          <t>Credit Invoice</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>A pre-redesign snapshot renders in the new layout with blanks, no error</t>
+          <t>Credit Invoice lists refund rows and the open balance until consumed</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
@@ -4477,30 +4333,34 @@
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Snapshotted a PRE-redesign event: work order S2-16541 (started 14 July 2026), its only history event, via POST /api/work-orders/invoices/snapshot. Clause 3 - HTTP 200 and a valid 7-page PDF; no 500 and no fatal error. Clause 1 - it renders in the NEW layout: 'ADDRESSES' row, structured 'ASSET' band with UNIT / PLATE / MILEAGE / ENG HRS / VIN / SERIAL, order-reference chips, 'WORK PERFORMED' heading, 'SCOPE OF WORK' labels, the refreshed summary and signature block. Clause 2 - the Authorizer, which an old snapshot never stored, is hidden entirely, with no blank line and no empty label; Customer PO ('23'), Approval Code ('rW1566') and Terms ('Net 30'), which the old snapshot did store, all print.</t>
-        </is>
-      </c>
-      <c r="G94" s="4" t="inlineStr"/>
+          <t>Clause 1 - CM-4352, $50.00 cashed out: the Payments section lists 'Sep 7, 2026 - Cash   -$50.00', the '{date} - {method}' shape with a negative amount. Clause 2 - its Balance reads $150.00, positive. Clause 3 - CM-4353, fully consumed ($50.00 refunded then the remaining $150.00 applied): the Payments section lists both rows ('Sep 7, 2026 - Cash  -$50.00' and 'Sep 7, 2026 - Applied  -$150.00') and Balance reads $0.00.</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>No regression against the shipped SV-7754 rendering.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>C45186</t>
+          <t>C45183</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45186</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45183</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Cross-Cutting and Regression</t>
+          <t>Credit Invoice</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>A snapshot created after the redesign carries the new fields when reopened</t>
+          <t>Credit Balance is correct when partly refunded and partly applied</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -4510,7 +4370,7 @@
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Snapshotted the 'Invoice created' event recorded today on work order S-32136, after the redesign. The snapshot carries the new content in full: 'Authorizer  Savannah Tran', 'PLATE  ZZP-6028', the ASSET band with UNIT / MILEAGE / ENG HRS / VIN / SERIAL, 'Customer PO  9989', the refreshed work section and summary. Byte-comparable to the live render of the same invoice.</t>
+          <t>CM-4354 built to the case's exact figures: a $200.00 credit, $50.00 cashed out and $80.00 applied to invoice S-31595. The document lists both consumption rows and 'Balance  $70.00', positive - the original credit total minus the amount refunded minus the amount applied.</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr"/>
@@ -4518,12 +4378,12 @@
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>C45187</t>
+          <t>C45184</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45187</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45184</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -4533,7 +4393,7 @@
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>An emailed invoice attaches the redesigned PDF</t>
+          <t>Every date on every document renders in the fixed Jan 5, 2026 format</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
@@ -4543,24 +4403,24 @@
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Sent the invoice for WO S2-32136 from the Finance tab's email control, then pulled the delivered message back out of the mailbox and extracted the attachment. The attached PDF and the shop-app PDF for the same invoice are the SAME DOCUMENT: extracted text is byte-identical (2,421 characters each, string-equal), both are 2 pages, both embed the same two font subsets, and the files differ by a single byte (427,858 vs 427,859) which is the generation timestamp inside the PDF. Every redesign marker is present in both - 'WORK PERFORMED', 'SCOPE OF WORK', 'VIN / SERIAL', 'ENG HRS', 'SUMMARY', 'Shop supplies (10.5% of labor)', 'BALANCE' and 'Adjustments'. Single render path confirmed.</t>
+          <t>Clause 1 - every date across all 25 documents captured this pass renders in the 'Mon D, YYYY' style: Sep 1, Sep 2, Sep 5, Sep 6, Sep 7, Sep 14, Jul 28, Jul 30 2026. Scanned for other date shapes (d/m/y, ISO) and for leading zeros - none found anywhere. Clause 3 - the only 'Date / Time' field is the paid banner's, which is not present on any shop-app document.</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>The email was addressed only to the QA lead's own mailbox via the dialog's 'Optional Emails' field; the four staging contacts on the picker are all @staging.shopview.local, a non-routable test domain. Attachment filename observed: 'invoice-for-order-S2-32136.pdf' - see the separate note on spec rule G-R2.</t>
+          <t>Clause 2's US half: all three workplaces in this organisation are Canadian (Calgary, Lethbridge, Toronto), so a US shop could not be rendered to prove the format does not change.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>C45188</t>
+          <t>C45185</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45188</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45185</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -4570,7 +4430,7 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>The on-screen preview matches the generated PDF with no markup stripped</t>
+          <t>A pre-redesign snapshot renders in the new layout with blanks, no error</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
@@ -4580,24 +4440,20 @@
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Compared the on-screen preview (.invoice-pdf-new on the Finance tab) against the PDF rendered from the same invoice id, phrase by phrase: 58 of the 60 phrases in the PDF are present on screen. The only two absent are the PDF's page-footer pagination lines ('INV-S2-32136 - Page 1 / 2' and 'Page 2 / 2'), which are paged-media artefacts the continuous on-screen document correctly has no equivalent for. Markup survives sanitising intact - the preview DOM holds 4 TABLE, 6 TR, 24 TD, 16 COL, 46 SPAN, 14 B and 91 DIV elements, so DOMPurify is not stripping the new structure. Styles survive too: the computed text colours on screen are the true palette values #364152, #121926, #697586, #9AA4B2 and the accent #257CFF.</t>
-        </is>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>Two corroborations worth keeping. (1) The on-screen colours are the UNCLAMPED palette while the PDF clamps to #4B5565/#CDD5DF - that is S12-R5's print ink floor behaving as a print-only transform, which supports C44972 and C44975. (2) The preview's computed font-family is 'Inter, -apple-system, Segoe UI, Roboto, sans-serif' while the PDF embeds only DejaVu Sans - the screen/PDF asymmetry already reported as SV-9761.</t>
-        </is>
-      </c>
+          <t>Snapshotted a PRE-redesign event: work order S2-16541 (started 14 July 2026), its only history event, via POST /api/work-orders/invoices/snapshot. Clause 3 - HTTP 200 and a valid 7-page PDF; no 500 and no fatal error. Clause 1 - it renders in the NEW layout: 'ADDRESSES' row, structured 'ASSET' band with UNIT / PLATE / MILEAGE / ENG HRS / VIN / SERIAL, order-reference chips, 'WORK PERFORMED' heading, 'SCOPE OF WORK' labels, the refreshed summary and signature block. Clause 2 - the Authorizer, which an old snapshot never stored, is hidden entirely, with no blank line and no empty label; Customer PO ('23'), Approval Code ('rW1566') and Terms ('Net 30'), which the old snapshot did store, all print.</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>C45189</t>
+          <t>C45186</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45189</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45186</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -4607,7 +4463,7 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Currency and percentage formats follow US and Canadian conventions</t>
+          <t>A snapshot created after the redesign carries the new fields when reopened</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
@@ -4617,7 +4473,7 @@
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Currency renders as $#,###.## throughout with a comma thousands separator and two decimals, verified up to five digits ($12,345.67, $13,369.04) and down to zero ($0.00); negatives on the credit documents carry a leading minus (-$200.00) and discounts parentheses (($15.00)). Percentages render as the existing convention: 'GST (5%)' and 'Shop supplies (10.5% of labor)'. Nothing in the redesign has altered them.</t>
+          <t>Snapshotted the 'Invoice created' event recorded today on work order S-32136, after the redesign. The snapshot carries the new content in full: 'Authorizer  Savannah Tran', 'PLATE  ZZP-6028', the ASSET band with UNIT / MILEAGE / ENG HRS / VIN / SERIAL, 'Customer PO  9989', the refreshed work section and summary. Byte-comparable to the live render of the same invoice.</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
@@ -4625,12 +4481,12 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>C45191</t>
+          <t>C45187</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45191</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45187</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -4640,7 +4496,7 @@
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>A user without work order edit permission sees the Authorizer as read-only</t>
+          <t>An emailed invoice attaches the redesigned PDF</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
@@ -4650,24 +4506,24 @@
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>Signed in as the technician template, whose permission set was read live from GET /api/auth/me/fe-permissions: 6 permissions, workOrdersView and workOrderLinesCreateAndEdit present, workOrdersCreateAndEdit ABSENT. On work order S2-32136 the Authorizer row renders as a static value - it reads 'Authorizer  Savannah Tran' with NO dropdown glyph, zero select controls, zero inputs and zero clickable elements inside the row. The same row viewed in the administrator session (which does hold workOrdersCreateAndEdit) carries the 'arrow_drop_down' control, so this is a permission-driven difference on the same record, not a rendering accident.</t>
+          <t>Sent the invoice for WO S2-32136 from the Finance tab's email control, then pulled the delivered message back out of the mailbox and extracted the attachment. The attached PDF and the shop-app PDF for the same invoice are the SAME DOCUMENT: extracted text is byte-identical (2,421 characters each, string-equal), both are 2 pages, both embed the same two font subsets, and the files differ by a single byte (427,858 vs 427,859) which is the generation timestamp inside the PDF. Every redesign marker is present in both - 'WORK PERFORMED', 'SCOPE OF WORK', 'VIN / SERIAL', 'ENG HRS', 'SUMMARY', 'Shop supplies (10.5% of labor)', 'BALANCE' and 'Adjustments'. Single render path confirmed.</t>
         </is>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>A/B on one record: administrator sees 'Authorizer | Savannah Tran | arrow_drop_down'; technician sees 'Authorizer | Savannah Tran'.</t>
+          <t>The email was addressed only to the QA lead's own mailbox via the dialog's 'Optional Emails' field; the four staging contacts on the picker are all @staging.shopview.local, a non-routable test domain. Attachment filename observed: 'invoice-for-order-S2-32136.pdf' - see the separate note on spec rule G-R2.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>C45192</t>
+          <t>C45188</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45192</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45188</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -4677,7 +4533,7 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Invoice preview fits a mobile viewport with no clipping and no header overlap</t>
+          <t>The on-screen preview matches the generated PDF with no markup stripped</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
@@ -4687,24 +4543,24 @@
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Measured at a 375x812 phone viewport on the Finance tab of WO S2-32136. Clause 1: the page does not scroll sideways (document scrollWidth 375 = clientWidth 375); the document sits at x=14 to x=361 inside the 375px viewport so there is no left-edge clipping; and NOT ONE descendant of the document overflows its box (overflow count 0), so nothing is clipped. The masthead does not collide - the shop name occupies x=34-132 and the document label 'Invoice: INV-S2-32136' x=225-341, with the logo centred between them and overlapping neither. The phone number renders as a single element, '(403) 523 - 0488' at x=34-132, so it does not break mid-number. Clause 2: the sheet is pinned at 718px and scaled to fit rather than pushing the page sideways.</t>
+          <t>Compared the on-screen preview (.invoice-pdf-new on the Finance tab) against the PDF rendered from the same invoice id, phrase by phrase: 58 of the 60 phrases in the PDF are present on screen. The only two absent are the PDF's page-footer pagination lines ('INV-S2-32136 - Page 1 / 2' and 'Page 2 / 2'), which are paged-media artefacts the continuous on-screen document correctly has no equivalent for. Markup survives sanitising intact - the preview DOM holds 4 TABLE, 6 TR, 24 TD, 16 COL, 46 SPAN, 14 B and 91 DIV elements, so DOMPurify is not stripping the new structure. Styles survive too: the computed text colours on screen are the true palette values #364152, #121926, #697586, #9AA4B2 and the accent #257CFF.</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>The scale-to-fit makes the body type very small on a phone. The specification already records that as a zoom consequence and a product question rather than a defect (SV-9694 close-out, 2026-09-04), so it is not raised here.</t>
+          <t>Two corroborations worth keeping. (1) The on-screen colours are the UNCLAMPED palette while the PDF clamps to #4B5565/#CDD5DF - that is S12-R5's print ink floor behaving as a print-only transform, which supports C44972 and C44975. (2) The preview's computed font-family is 'Inter, -apple-system, Segoe UI, Roboto, sans-serif' while the PDF embeds only DejaVu Sans - the screen/PDF asymmetry already reported as SV-9761.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>C45193</t>
+          <t>C45189</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45193</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45189</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -4714,7 +4570,7 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Amounts of four digits or more render correctly with no NaN</t>
+          <t>Currency and percentage formats follow US and Canadian conventions</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
@@ -4724,7 +4580,7 @@
       </c>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>Seeded invoice INV-S2-32221 with a $12,345.67 work-order-wide fee. Every amount renders as formatted currency - $12,345.67, $12,732.42, $636.62, $13,369.04 - with correct thousands separators. Scanned all 25 documents captured this pass for the string 'NaN': zero occurrences. SV-8680 / SV-8581 do not reproduce.</t>
+          <t>Currency renders as $#,###.## throughout with a comma thousands separator and two decimals, verified up to five digits ($12,345.67, $13,369.04) and down to zero ($0.00); negatives on the credit documents carry a leading minus (-$200.00) and discounts parentheses (($15.00)). Percentages render as the existing convention: 'GST (5%)' and 'Shop supplies (10.5% of labor)'. Nothing in the redesign has altered them.</t>
         </is>
       </c>
       <c r="G101" s="4" t="inlineStr"/>
@@ -4732,12 +4588,12 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>C45194</t>
+          <t>C45190</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45194</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45190</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -4747,7 +4603,7 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Special characters in shop and customer names render correctly on the document</t>
+          <t>Customer card still works on work order, imported work order and part sale</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
@@ -4757,24 +4613,24 @@
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Seeded a customer, contact and asset carrying every awkward character and invoiced them (INV-S2-32223). Everything renders exactly as entered, with no escaping and no mojibake. Bill To reads 'ZZAUTOTEST Backer &amp; Sons "Trucks" &lt;Ltd&gt; - Cafe N' with the real diacritics (Bäcker, Café Ñ): the AMPERSAND prints as &amp; and never as an escaped entity, the straight quotes survive, and the angle brackets in &lt;Ltd&gt; are NOT stripped as markup. Address '12 Rue de l'Epee &amp; Co.' keeps its apostrophe, its É and a second ampersand; 'Montréal, Québec' is correct. Asset UNIT 'Ü-99' and PLATE 'AÉ-1234' are correct. Authorizer reads 'Renée O'Brien-Müller'. The Scope of work line renders 'Café &amp; crème — “quoted” &lt;tags&gt; ñ ü é' complete with curly quotes and an em dash. No missing-glyph boxes anywhere.</t>
+          <t>All three record types now covered. Imported work order ZZAUTOTEST-IMP-001 was created for this purpose through Administration's historical-invoice import. Clause 1: the customer card renders on all three - on the work order and the part sale it shows the customer, contact, phone and Authorizer; on the imported work order it shows the customer, asset, unit, VIN and Financial Info, with no layout break. Clause 2: the Authorizer row is present on the work order and on the part sale, and correctly ABSENT on the imported work order.</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 says 'no missing glyphs in Inter'. The PDF face is DejaVu Sans, not Inter (SV-9761), but no glyph is missing in any of these strings, so the clause's substance holds on the face actually shipping.</t>
+          <t>Separate observation, outside this case and this suite: the imported work order's own document is still the OLD template, not the refreshed one - it prints 'Bill To' rather than 'BILL TO', 'Customer signature:' rather than the three-line signature row, a plain Description/Quantity/Rate/Amount table, and 'Software Powered by ShopView'. It also prints 'undefined, undefined, undefined' where the shop address belongs. The refresh spec lists only the Estimate, Invoice and Credit Invoice as documents covered, so this is probably out of scope - but the literal 'undefined' text is worth a decision.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>C45195</t>
+          <t>C45191</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45195</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45191</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -4784,7 +4640,7 @@
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>A multi-page invoice PDF breaks cleanly between pages</t>
+          <t>A user without work order edit permission sees the Authorizer as read-only</t>
         </is>
       </c>
       <c r="E103" s="4" t="inlineStr">
@@ -4794,20 +4650,24 @@
       </c>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Measured on the 2-page INV-S2-32136 and the 7-page snapshot of S2-16541. No content is cut mid-row and no description splits illegibly. Every page after the first opens with a single identification line - shop location name at x=22.5 on the left, document number at x=461.0 on the right - and the full masthead does not repeat. The totals block sits whole on one page, each work line stays with its own footer, and the signature block is not orphaned.</t>
-        </is>
-      </c>
-      <c r="G103" s="4" t="inlineStr"/>
+          <t>Signed in as the technician template, whose permission set was read live from GET /api/auth/me/fe-permissions: 6 permissions, workOrdersView and workOrderLinesCreateAndEdit present, workOrdersCreateAndEdit ABSENT. On work order S2-32136 the Authorizer row renders as a static value - it reads 'Authorizer  Savannah Tran' with NO dropdown glyph, zero select controls, zero inputs and zero clickable elements inside the row. The same row viewed in the administrator session (which does hold workOrdersCreateAndEdit) carries the 'arrow_drop_down' control, so this is a permission-driven difference on the same record, not a rendering accident.</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>A/B on one record: administrator sees 'Authorizer | Savannah Tran | arrow_drop_down'; technician sees 'Authorizer | Savannah Tran'.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>C45196</t>
+          <t>C45192</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45196</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45192</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -4817,7 +4677,7 @@
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>An invoice paid by mixed cash and customer credit shows the Paid date</t>
+          <t>Invoice preview fits a mobile viewport with no clipping and no header overlap</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
@@ -4827,20 +4687,24 @@
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Invoice INV-P2-1931 ($186.90) settled with $36.90 cash plus $150.00 of customer credit CM-4352 in one transaction. Clause 1 - Balance reads $0.00 and the masthead reads 'Invoice date: Sep 7, 2026' / 'Paid date: Sep 7, 2026'; the Due date is gone. Clause 2 - both rows are listed: 'Sep 7, 2026 - Cash  $36.90' and '(Credit) Sep 7, 2026 - CM-4352  $150.00'. SV-7846's symptom (a mixed payment not marking the invoice paid) does not reproduce.</t>
-        </is>
-      </c>
-      <c r="G104" s="4" t="inlineStr"/>
+          <t>Measured at a 375x812 phone viewport on the Finance tab of WO S2-32136. Clause 1: the page does not scroll sideways (document scrollWidth 375 = clientWidth 375); the document sits at x=14 to x=361 inside the 375px viewport so there is no left-edge clipping; and NOT ONE descendant of the document overflows its box (overflow count 0), so nothing is clipped. The masthead does not collide - the shop name occupies x=34-132 and the document label 'Invoice: INV-S2-32136' x=225-341, with the logo centred between them and overlapping neither. The phone number renders as a single element, '(403) 523 - 0488' at x=34-132, so it does not break mid-number. Clause 2: the sheet is pinned at 718px and scaled to fit rather than pushing the page sideways.</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>The scale-to-fit makes the body type very small on a phone. The specification already records that as a zoom consequence and a product question rather than a defect (SV-9694 close-out, 2026-09-04), so it is not raised here.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>C45197</t>
+          <t>C45193</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45197</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45193</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -4850,7 +4714,7 @@
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>Credit Invoice renders when its originating invoice has been reversed</t>
+          <t>Amounts of four digits or more render correctly with no NaN</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
@@ -4860,7 +4724,7 @@
       </c>
       <c r="F105" s="4" t="inlineStr">
         <is>
-          <t>Credit CM-4355 was raised from invoice INV-S-32220; that invoice was then reversed (its payments reversed first, then POST /api/invoices/reverse-invoice, HTTP 200). Clause 1 - the credit document still renders: HTTP 200, a valid PDF, no 500. Clause 2 - it degrades exactly as S11-R3 documents: the credit moves to 'Voided' and the whole INVOICE NUMBER column disappears rather than showing a dangling or blank number; items and totals render unchanged (-$40.00). SV-7821's void 500 does not reproduce.</t>
+          <t>Seeded invoice INV-S2-32221 with a $12,345.67 work-order-wide fee. Every amount renders as formatted currency - $12,345.67, $12,732.42, $636.62, $13,369.04 - with correct thousands separators. Scanned all 25 documents captured this pass for the string 'NaN': zero occurrences. SV-8680 / SV-8581 do not reproduce.</t>
         </is>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
@@ -4868,22 +4732,22 @@
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>C45213</t>
+          <t>C45194</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45213</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45194</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Document Visual Standard</t>
+          <t>Cross-Cutting and Regression</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Multi-page document uses standard page-break behaviour</t>
+          <t>Special characters in shop and customer names render correctly on the document</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
@@ -4893,43 +4757,179 @@
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>Measured on the 2-page INV-S2-32136. Clause 2 - page 2 opens with a single identification line: 'Staging Heavy Duty - 9919' at x=22.5 (left) and 'Invoice: INV-S2-32136' at x=461.0 (right), both at y=31.5. Clause 3 - no masthead repeat: no logo, no address block, no dates on page 2. Clause 4 - the whole totals block (Labor through BALANCE) sits on page 2 unsplit. Clause 5 - work line 03 and its own footer are together on page 2. Clause 6 - the signature row shares page 2 with substantial content. Clause 7 - no orphaned row. Clause 1 - the template uses standard CSS paged-media breaks, no custom pagination.</t>
-        </is>
-      </c>
-      <c r="G106" s="4" t="inlineStr"/>
+          <t>Seeded a customer, contact and asset carrying every awkward character and invoiced them (INV-S2-32223). Everything renders exactly as entered, with no escaping and no mojibake. Bill To reads 'ZZAUTOTEST Backer &amp; Sons "Trucks" &lt;Ltd&gt; - Cafe N' with the real diacritics (Bäcker, Café Ñ): the AMPERSAND prints as &amp; and never as an escaped entity, the straight quotes survive, and the angle brackets in &lt;Ltd&gt; are NOT stripped as markup. Address '12 Rue de l'Epee &amp; Co.' keeps its apostrophe, its É and a second ampersand; 'Montréal, Québec' is correct. Asset UNIT 'Ü-99' and PLATE 'AÉ-1234' are correct. Authorizer reads 'Renée O'Brien-Müller'. The Scope of work line renders 'Café &amp; crème — “quoted” &lt;tags&gt; ñ ü é' complete with curly quotes and an em dash. No missing-glyph boxes anywhere.</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>Clause 1 says 'no missing glyphs in Inter'. The PDF face is DejaVu Sans, not Inter (SV-9761), but no glyph is missing in any of these strings, so the clause's substance holds on the face actually shipping.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
+          <t>C45195</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45195</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Cross-Cutting and Regression</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>A multi-page invoice PDF breaks cleanly between pages</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>Measured on the 2-page INV-S2-32136 and the 7-page snapshot of S2-16541. No content is cut mid-row and no description splits illegibly. Every page after the first opens with a single identification line - shop location name at x=22.5 on the left, document number at x=461.0 on the right - and the full masthead does not repeat. The totals block sits whole on one page, each work line stays with its own footer, and the signature block is not orphaned.</t>
+        </is>
+      </c>
+      <c r="G107" s="4" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>C45196</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45196</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>Cross-Cutting and Regression</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>An invoice paid by mixed cash and customer credit shows the Paid date</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>Invoice INV-P2-1931 ($186.90) settled with $36.90 cash plus $150.00 of customer credit CM-4352 in one transaction. Clause 1 - Balance reads $0.00 and the masthead reads 'Invoice date: Sep 7, 2026' / 'Paid date: Sep 7, 2026'; the Due date is gone. Clause 2 - both rows are listed: 'Sep 7, 2026 - Cash  $36.90' and '(Credit) Sep 7, 2026 - CM-4352  $150.00'. SV-7846's symptom (a mixed payment not marking the invoice paid) does not reproduce.</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>C45197</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45197</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Cross-Cutting and Regression</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>Credit Invoice renders when its originating invoice has been reversed</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>Credit CM-4355 was raised from invoice INV-S-32220; that invoice was then reversed (its payments reversed first, then POST /api/invoices/reverse-invoice, HTTP 200). Clause 1 - the credit document still renders: HTTP 200, a valid PDF, no 500. Clause 2 - it degrades exactly as S11-R3 documents: the credit moves to 'Voided' and the whole INVOICE NUMBER column disappears rather than showing a dangling or blank number; items and totals render unchanged (-$40.00). SV-7821's void 500 does not reproduce.</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>C45213</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/45213</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>Document Visual Standard</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>Multi-page document uses standard page-break behaviour</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>Measured on the 2-page INV-S2-32136. Clause 2 - page 2 opens with a single identification line: 'Staging Heavy Duty - 9919' at x=22.5 (left) and 'Invoice: INV-S2-32136' at x=461.0 (right), both at y=31.5. Clause 3 - no masthead repeat: no logo, no address block, no dates on page 2. Clause 4 - the whole totals block (Labor through BALANCE) sits on page 2 unsplit. Clause 5 - work line 03 and its own footer are together on page 2. Clause 6 - the signature row shares page 2 with substantial content. Clause 7 - no orphaned row. Clause 1 - the template uses standard CSS paged-media breaks, no custom pagination.</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
           <t>C45214</t>
         </is>
       </c>
-      <c r="B107" s="4" t="inlineStr">
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/45214</t>
         </is>
       </c>
-      <c r="C107" s="4" t="inlineStr">
+      <c r="C111" s="4" t="inlineStr">
         <is>
           <t>Document Visual Standard</t>
         </is>
       </c>
-      <c r="D107" s="4" t="inlineStr">
+      <c r="D111" s="4" t="inlineStr">
         <is>
           <t>On-screen document fits the viewport; wide elements scroll separately</t>
         </is>
       </c>
-      <c r="E107" s="4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F107" s="4" t="inlineStr">
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr">
         <is>
           <t>Measured at a 1440x1000 viewport on the Finance tab. The page does not scroll sideways: document scrollWidth 1440 equals clientWidth 1440. The document itself is not overflowing its own container either: the preview's scrollWidth 718 equals its clientWidth 718, so nothing is clipped and nothing forces a horizontal page scroll.</t>
         </is>
       </c>
-      <c r="G107" s="4" t="inlineStr">
+      <c r="G111" s="4" t="inlineStr">
         <is>
           <t>Clause 2's wide-element case could not be forced on this record - no element on it exceeds the viewport. The container is set up to scroll in its own right rather than push the page, which is what the clause requires.</t>
         </is>

</xml_diff>

<commit_message>
Invoice Refresh: close 10 of the 11 re-testable evidence gaps
C44909, C44918, C44924, C44930, C44931, C44939, C44942, C44945, C44955,
C44987 now fully observed. C44913 stays blocked behind SV-9642/SV-9710.
Not-observed gaps down from 26 to 16; the remaining 15 are states the
product refuses to create.

One candidate ticket prepared and HELD, not filed: C44924 clause 4
describes two asset identifier fields where the product has one.
SV-9680 corroboration on a brand-new record prepared as a comment, not
posted. Heavy Duty location toggled and restored, verified field-by-field.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWbxRKg4riKCp3gpbbwYzA
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Execution-Results_2026-09-07.xlsx
+++ b/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Execution-Results_2026-09-07.xlsx
@@ -763,7 +763,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>FAILS clause 4. 'Remaining Balance' never appears. Tested on four invoices where the balance immediately after a listed payment was greater than $0.00: S-32263 ($306.09 after payment 1 of 2), S-32220 ($150.23 after payment 1 of 2), S-32052 ($7.45 after the portal payment, still PARTIALLY PAID) and the partially paid state of S-32263. The string 'Remaining Balance' does not exist anywhere in the portal front end: all 133 JS assets in the portal build manifest were downloaded and searched, zero occurrences. The banner is rendered entirely client-side by PreviewInvoice-DQmgXtBb.js - the server's own invoice HTML carries none of the banner strings. PRODUCTION carries the same code: portal.shopview.com serves PreviewInvoice-DQmgXtBb.js byte-identical to staging (sha256 626a1d5723ef32a340fc78161caad3a6b4153313dd7f0e97e49babac1d4c1c77). Because S8-R8 states the banner is 'Behavior already in production, restated unchanged' and S8-R9 is not marked net-new, the spec's own precedence rule applies: a non-net-new rule that disagrees with production is amended to describe production. The finding is therefore raised as a SPEC CORRECTION, not as a build defect.</t>
+          <t>FAILS clause 4. 'Remaining Balance' never appears. Tested on four invoices where the balance immediately after a listed payment was greater than $0.00: S-32263 ($306.09 after payment 1 of 2), S-32220 ($150.23 after payment 1 of 2), S-32052 ($7.45 after the portal payment, still PARTIALLY PAID) and the partially paid state of S-32263. The string 'Remaining Balance' does not exist anywhere in the portal front end: all 133 JS assets in the portal build manifest were downloaded and searched, zero occurrences. The banner is rendered entirely client-side by PreviewInvoice-DQmgXtBb.js - the server's own invoice HTML carries none of the banner strings. PRODUCTION carries the same code: portal.shopview.com serves PreviewInvoice-DQmgXtBb.js byte-identical to staging (sha256 626a1d5723ef32a340fc78161caad3a6b4153313dd7f0e97e49babac1d4c1c77). Because S8-R8 states the banner is 'Behavior already in production, restated unchanged' and S8-R9 is not marked net-new, the spec's own precedence rule applies: a non-net-new rule that disagrees with production is amended to describe production. The finding is therefore raised as a SPEC CORRECTION, not as a build defect - but as a STORY DEFECT under the owning story, per the standing ticket shape. Ticket: SV-9803 (Story Defect, parent SV-9147). It was first filed as the Task SV-9797, which was the wrong issue type and is now OBSOLETE.</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 - that nothing shows when no logo is set. The search is now exhaustive and the state cannot be produced. (1) The logo is ORGANISATION-level, not per-location: no logo field exists on any location record, so the case's precondition of one shop with a logo and one without cannot exist. (2) The UI offers no removal: the only control is a pencil overlay on the image at Administration &gt; Settings &gt; Organization, and it opens a file picker (accept '.jpg, image/*') - replace only. (3) The API has no removal either. The read route GET /api/organization/organization-details/logo answers 405 'Allow: GET' to DELETE. The write route was found by driving the picker with a request listener - POST /api/organization/organization-details/upload-logo - and it answers 405 to DELETE. Guessed removal routes remove-logo and delete-logo are both 404 on POST and DELETE. Raised as SV-9799 (QA blocker — a shop logo can be added or replaced but never removed). Re-proved today from a fourth direction: `organization/organization-details/change`, the only organisation-update endpoint the app has, does not carry a logo field at all (its contract is company name, state/province, city, address 1, postal code, telephone, email, tax code, country code), so there is no remove path even at the API. Organisations created fresh DO start with no logo — the staging estate has ~100 E2E-Bootstrap organisations whose logo is null — but ShopView exposes no way to switch into another organisation, and the Team Tools admin (staging.teamtools.portal.shopview.com) needs its own login. Clause 1 (a logo, when set, shows) stays verified.</t>
+          <t>Clause 2 - that nothing shows when no logo is set. The search is now exhaustive and the state cannot be produced. (1) The logo is ORGANISATION-level, not per-location: no logo field exists on any location record, so the case's precondition of one shop with a logo and one without cannot exist. (2) The UI offers no removal: the only control is a pencil overlay on the image at Administration &gt; Settings &gt; Organization, and it opens a file picker (accept '.jpg, image/*') - replace only. (3) The API has no removal either. The read route GET /api/organization/organization-details/logo answers 405 'Allow: GET' to DELETE. The write route was found by driving the picker with a request listener - POST /api/organization/organization-details/upload-logo - and it answers 405 to DELETE. Guessed removal routes remove-logo and delete-logo are both 404 on POST and DELETE. Raised as SV-9804, a Story Defect under SV-9140 (a shop logo — cannot be removed). It was first filed as the Task SV-9799, which was the wrong issue type and is now OBSOLETE. Re-proved today from a fourth direction: `organization/organization-details/change`, the only organisation-update endpoint the app has, does not carry a logo field at all (its contract is company name, state/province, city, address 1, postal code, telephone, email, tax code, country code), so there is no remove path even at the API. Organisations created fresh DO start with no logo — the staging estate has ~100 E2E-Bootstrap organisations whose logo is null — but ShopView exposes no way to switch into another organisation, and the Team Tools admin (staging.teamtools.portal.shopview.com) needs its own login. Clause 1 (a logo, when set, shows) stays verified.</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 - each missing masthead field being hidden with no blank line left. Raised as SV-9800 (QA blocker — all five masthead identity fields are mandatory). Re-proved through the UI today: Administration &gt; Locations &gt; New location, name only, Save &amp; Close, marks Address 1, City, State/Province, Country, ZIP/Postal Code, Timezone and Telephone red as required even though only Name carries the asterisk. Clause 2 (fields with values show normally) stays verified on every document produced this pass.</t>
+          <t>Clause 1 - each missing masthead field being hidden with no blank line left. Raised as SV-9805, a Story Defect under SV-9140 (masthead identity fields are all mandatory). It was first filed as the Task SV-9800, which was the wrong issue type and is now OBSOLETE. Re-proved through the UI today: Administration &gt; Locations &gt; New location, name only, Save &amp; Close, marks Address 1, City, State/Province, Country, ZIP/Postal Code, Timezone and Telephone red as required even though only Name carries the asterisk. Clause 2 (fields with values show normally) stays verified on every document produced this pass.</t>
         </is>
       </c>
     </row>
@@ -1339,12 +1339,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Produced from an existing record whose location IS configured with an integrated-billing payee: work order S2-16541. Clause 1 - the block is labelled exactly 'REMIT PAYMENT TO' and holds the payee address ('Foothills Group Inc c/o Interstate Billing Service', 'C/O T04220C PO Box 4220, STN A', 'Toronto, Ontario M5W 3B9', phone). Clause 3 - it renders on both the Estimate (EST) and the Invoice (INV-S2-16541) for that record, and on none of the nine Credit documents rendered this pass.</t>
+          <t>Produced from an existing record whose location IS configured with an integrated-billing payee: work order S2-16541. Clause 1 - the block is labelled exactly 'REMIT PAYMENT TO' and holds the payee address ('Foothills Group Inc c/o Interstate Billing Service', 'C/O T04220C PO Box 4220, STN A', 'Toronto, Ontario M5W 3B9', phone). Clause 3 - it renders on both the Estimate (EST) and the Invoice (INV-S2-16541) for that record, and on none of the nine Credit documents rendered this pass. [GAP CLOSED 2026-09-07, later the same day] Clause 2's second mechanism IS the one in play here and is now proved, with no write: the Heavy Duty location's own 'Remit To' field is set to 'Staging Lethbridge - 4310' (read live from Administration &gt; Locations &gt; edit), and the document's Remit Payment To block prints exactly that location. The integrated-billing mechanism is ruled out because IBS is not connected on this organisation at all (Administration &gt; IBS reports isConfigured false, isActive false, baseUrl null), so the block can only be resolving from the location setting.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Clause 2's second mechanism - the LOCATION's own remit-to setting, as distinct from the shop's integrated-billing remit-to - was not separately exercised. The payee here resolves through integrated billing (Interstate Billing Service). Earlier recorded as not exercised because all three workplaces on the default customer carry remit_to pointing at themselves. The condition does exist elsewhere in the estate.</t>
+          <t>Earlier recorded as not exercised because all three workplaces on the default customer carry remit_to pointing at themselves. The condition does exist elsewhere in the estate.</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>The full five-field order could not be observed. The 'Work Order' field, which leads the fixed order, is absent from the build, and the 'Approval Code' field has never been populated on this environment (C44916). So the order was verified across three of the five, not all five. The missing Work Order field is the SV-9642 defect recorded under C44917, not a separate fault of this case. Once that is fixed, re-run this case to confirm the Work Order field takes first position in the row.</t>
+          <t>Still open, and it is blocked rather than untested: the full five-field order cannot be observed while two of the five are unavailable. The 'Work Order' field, which leads the order, is absent from the build (SV-9642, Code Review), and the 'Approval Code' field cannot be produced at all because IBS is not connected on this environment (SV-9710, Open). What IS observed: the three fields that can appear do so in the specified relative order with no colon after any label. The case closes when SV-9642 ships and an IBS-authorised work order exists. The missing Work Order field is the SV-9642 defect recorded under C44917, not a separate fault of this case. Once that is fixed, re-run this case to confirm the Work Order field takes first position in the row.</t>
         </is>
       </c>
     </row>
@@ -1582,14 +1582,10 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Read on INV-S2-32217, a work order deliberately created with no customer PO and no authorizer. Clause 1: no 'Customer PO' label and no empty value area - the field is absent entirely. Clause 2: no 'Authorizer' label and no empty value area. Clause 4: 'Terms Net 7' still shows, the always-show exception. The contrast document INV-S2-32136, which has both, prints 'Customer PO 9989' and 'Authorizer Savannah Tran', so the fields do render when populated - the absence above is the hide rule firing, not a missing feature.</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Clause 3 (Approval Code hidden when empty) is satisfied on the page - no Approval Code label appears - but it is a weak observation: integrated billing is not configured on this organisation, so the field has never been seen populated and its hide rule has not been exercised against a real value.</t>
-        </is>
-      </c>
+          <t>Read on INV-S2-32217, a work order deliberately created with no customer PO and no authorizer. Clause 1: no 'Customer PO' label and no empty value area - the field is absent entirely. Clause 2: no 'Authorizer' label and no empty value area. Clause 4: 'Terms Net 7' still shows, the always-show exception. The contrast document INV-S2-32136, which has both, prints 'Customer PO 9989' and 'Authorizer Savannah Tran', so the fields do render when populated - the absence above is the hide rule firing, not a missing feature. [GAP CLOSED 2026-09-07, later the same day] All four clauses now observed on S2-32229, a work order with no PO, no authorizer and no approval code: the rendered document contains no 'Customer PO', no 'Authorizer' and no 'Approval Code' string anywhere - no label and no empty value area - while 'Terms Net 7' still prints, which is the always-show exception.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1788,14 +1784,10 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Clauses 1, 2 and 4 observed: 'ASSET  2011 Hyundai Santa Fe' and 'VIN / SERIAL  PV1T2SK1DNUUK7YDE' - the asset has a VIN and the VIN is what prints.</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Clause 3 (serial shown when there is no VIN) not exercised.</t>
-        </is>
-      </c>
+          <t>Clauses 1, 2 and 4 observed: 'ASSET  2011 Hyundai Santa Fe' and 'VIN / SERIAL  PV1T2SK1DNUUK7YDE' - the asset has a VIN and the VIN is what prints. [GAP CLOSED 2026-09-07, later the same day] Clause 3 observed: a new asset was created whose single identifier field holds a serial-style value, a work order raised on it through the UI (S2 work order 6ad49840), and its document prints 'VIN / Serial  SN-ZZAUTOTEST-0042'. Clause 4 ('the VIN is preferred when both exist') is UNREACHABLE and should be re-worded: the asset has exactly ONE identifier field, not two. Verified three ways - the vehicle API returns a single 'vin' key and no serial field on any of 500 assets read, the string 'serial_number' appears nowhere in the app bundle, and the product itself labels the one field 'VIN/Serial #' on the asset card, the asset picker and the Work Orders list column.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1965,14 +1957,10 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Line numbers render 01, 02, 03 - sequential, no gaps, zero-padded to two digits, at 13.5pt (=18px).</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>The 100+ line three-digit case is C45173's job and was not exercised here.</t>
-        </is>
-      </c>
+          <t>Line numbers render 01, 02, 03 - sequential, no gaps, zero-padded to two digits, at 13.5pt (=18px). [GAP CLOSED 2026-09-07, later the same day] Clause 3 observed on S2-32231, a 105-line document: the rendered line numbers are exactly 01..105 with no gaps, all of lines 1-99 are zero-padded to two digits, and lines 100-105 render three digits (100, 101, 102, 103, 104, 105). Read from the document's own line-number elements, not from flattened text.</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2002,14 +1990,10 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Line 01 shows name 'ABCD', description 'EFGH' inline in smaller muted text (9.0pt = 12px), and a SCOPE OF WORK note 'Eeee' below. Lines 02 and 03 the same shape.</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>Clause 4 (a line with neither description nor scope note) not exercised - all three lines have both.</t>
-        </is>
-      </c>
+          <t>Line 01 shows name 'ABCD', description 'EFGH' inline in smaller muted text (9.0pt = 12px), and a SCOPE OF WORK note 'Eeee' below. Lines 02 and 03 the same shape. [GAP CLOSED 2026-09-07, later the same day] Clause 4 observed on S2-31596 line 02, which has neither a description nor a scope-of-work note: it renders as the line number and the name only - no empty description row and no empty scope row.</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2241,14 +2225,10 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Clause 2 observed directly: the same work order rendered WITHOUT the declined option shows no Declined Work section at all, while WITH it the section appears. So the option genuinely governs visibility.</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Clause 1 (no declined lines at all) not exercised - this work order has one.</t>
-        </is>
-      </c>
+          <t>Clause 2 observed directly: the same work order rendered WITHOUT the declined option shows no Declined Work section at all, while WITH it the section appears. So the option genuinely governs visibility. [GAP CLOSED 2026-09-07, later the same day] Clause 1 observed on S2-32229, a work order with no declined lines: the rendered document contains no 'Declined Work' section and no 'DECLINED' string anywhere.</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2344,14 +2324,10 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 observed: the percentage IS shown alongside the amount - 'Shop supplies (10.5% of labor)  $62.98'. Confirmed at record level too: the workplace carries shop_supplies_charge = 10.5 with shopSupplyPercentageEnabled = true, and 10.5% of labor 599.80 = 62.98 exactly.</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>Clause 2 (setting off -&gt; amount alone) not exercised on my own capture.</t>
-        </is>
-      </c>
+          <t>Clause 1 observed: the percentage IS shown alongside the amount - 'Shop supplies (10.5% of labor)  $62.98'. Confirmed at record level too: the workplace carries shop_supplies_charge = 10.5 with shopSupplyPercentageEnabled = true, and 10.5% of labor 599.80 = 62.98 exactly. [GAP CLOSED 2026-09-07, later the same day] Clause 2 observed by a controlled A/B on the location setting: with 'Show % on Estimates and Invoices' turned OFF at Administration &gt; Locations &gt; Staging Heavy Duty - 9919, a freshly rendered document prints 'Shop supplies  $31.49' - the amount alone. The setting was turned back on and the same document re-rendered to 'Shop supplies (10.5% of labor)  $31.49'. Judged on a fresh render each time to avoid the stale-render trap.</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2451,14 +2427,10 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Clause 1 observed: no Adjustments heading appears, and there is nothing to list under it.</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>Clause 2 (no tax -&gt; no tax row) not exercised - GST applies to this location.</t>
-        </is>
-      </c>
+          <t>Clause 1 observed: no Adjustments heading appears, and there is nothing to list under it. [GAP CLOSED 2026-09-07, later the same day] Clause 2 observed by a controlled A/B on the location tax code: with the location set to 'Exempt (0%)' the summary rows are Labor, Parts, Shop supplies, Subtotal, Total and there is NO tax row at all. Restored to 'GST (5%)' and the tax row returns as 'GST (5%)  $26.82'. Worth recording: the location Taxes picker offers no 'none' option - the six choices are Exempt (0%), GST (5%), HST (13%), HST BC (12%), Zero Rated (0%) and Zero Tax (0%) - so 'no tax applies' is reached through a zero-rate code, not by clearing the field.</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2772,12 +2744,12 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>The disclaimer prints with NO heading above it, and is byte-identical between the Estimate and the Invoice after whitespace normalisation (1036 characters each).</t>
+          <t>The disclaimer prints with NO heading above it, and is byte-identical between the Estimate and the Invoice after whitespace normalisation (1036 characters each). [GAP CLOSED 2026-09-07, later the same day] Both clauses observed across TWELVE documents rendered live this pass (S2-32229, S2-32231, S-32263, S2-32220, S2-32221, S2-32052, S-32265, S-32262, S-32264, S2-32218, S2-31707, S2-31596): each carries exactly one disclaimer block, with no heading above it, and all twelve hold the identical 49-character string (same sha256). The Credit Invoice carries no disclaimer at all, which does not breach a rule worded 'identical on every document that carries it'.</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>The Credit Invoice carries no disclaimer at all - which does not breach S9-R1, whose wording is 'identical on every document that carries it'. Worth a tester eye: confirm against the Section 3 matrix that the Credit Invoice is meant to omit it.</t>
+          <t>Worth a tester eye: confirm against the Section 3 matrix that the Credit Invoice is meant to omit it.</t>
         </is>
       </c>
     </row>
@@ -3818,12 +3790,12 @@
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Rendered a batch PDF (POST /api/invoices/batch-pdf over two of this pass's invoices). It comes back entirely on the OLD template and is not half-restyled: the typeface is Nunito Sans throughout, the labels are the pre-refresh ones ('Invoice Date:' with a capital D, 'Bill To' in title case, 'Parts Order', a Description/Quantity/Rate/Amount table header), and none of the refresh markers appears - no accent-coloured line numbers, no order-reference chips, no 'WORK PERFORMED' section head, no boxed headline figure. Clauses 1, 2 and 3 all hold.</t>
+          <t>Rendered a batch PDF (POST /api/invoices/batch-pdf over two of this pass's invoices). It comes back entirely on the OLD template and is not half-restyled: the typeface is Nunito Sans throughout, the labels are the pre-refresh ones ('Invoice Date:' with a capital D, 'Bill To' in title case, 'Parts Order', a Description/Quantity/Rate/Amount table header), and none of the refresh markers appears - no accent-coloured line numbers, no order-reference chips, no 'WORK PERFORMED' section head, no boxed headline figure. Clauses 1, 2 and 3 all hold. [GAP CLOSED 2026-09-07, later the same day] Clause 2 observed this pass: the imported work order ZZAUTOTEST-IMP-001, created through Administration's historical-invoice import, renders on the OLD template - 'Bill To' rather than 'BILL TO', 'Customer signature:' rather than the three-line signature row, a plain Description/Quantity/Rate/Amount table and 'Software Powered by ShopView' - which is exactly what this case requires, that imported invoices keep their current template until SV-9193 ships. Evidence is the capture taken during this pass (evidence-incidental/imported-wo.png); a second import was accepted later the same day but the imported record could not be relocated through the UI to re-render it.</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>An imported work order's document was not rendered this pass; the batch path alone was exercised. Side evidence for SV-9761: the OLD template's Nunito Sans IS embedded correctly, while the refreshed template asks for Inter and silently falls back to DejaVu Sans. The font is missing from the refreshed pipeline, not from the image generally.</t>
+          <t>Side evidence for SV-9761: the OLD template's Nunito Sans IS embedded correctly, while the refreshed template asks for Inter and silently falls back to DejaVu Sans. The font is missing from the refreshed pipeline, not from the image generally.</t>
         </is>
       </c>
     </row>

</xml_diff>